<commit_message>
REV2: ventilador axial mural Ø560 mm por uniformidad con montaje típico de planta
- HD-VENT-001: axial mural (placa mural) Ø560 mm transmisión directa; montaje
  con estructura de unión pernada, cubierta intemperie y malla de protección
  interior; motor encapsulado severe duty en la corriente de aire.
- HD-FILT-001: banco de filtración MERV 8 + MERV 13-14 dentro de la cubierta
  intemperie; eliminadas caja/housing, transición cuadrado/circular y flexible.
- listado_equipos.md: nuevos ítems cubierta (9), estructura de unión (8) y
  malla de protección interior (10); eliminados flexible y caja/housing.
- bases_diseno.yaml (rev 2), generar_excel.py (filas ventilador seleccionado
  Ø560, v_boca real 4,33 m/s), INF-001/INF-002 LaTeX, informe_investigacion.md.
- Imagen de referencia DTS-001 = Montaje/DISENOFINAL.png; croquis obsoleto
  eliminado; docs/index.html actualizado.
- Emitidos 7 entregables + PDF alternativo DTS-001; contexto y vault.
</commit_message>
<xml_diff>
--- a/Emisiones/2.0 HV-MEMORIAS DE CALCULO/P2437-HV-CAL-001.xlsx
+++ b/Emisiones/2.0 HV-MEMORIAS DE CALCULO/P2437-HV-CAL-001.xlsx
@@ -3767,7 +3767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O144"/>
+  <dimension ref="A1:O150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30.6" customWidth="1" min="1" max="1"/>
@@ -3846,10 +3846,10 @@
     <col width="13" customWidth="1" min="82" max="82"/>
     <col width="13" customWidth="1" min="83" max="83"/>
     <col width="13" customWidth="1" min="84" max="84"/>
+    <col width="13" customWidth="1" min="85" max="85"/>
     <col width="13" customWidth="1" min="86" max="86"/>
-    <col width="13" customWidth="1" min="88" max="88"/>
+    <col width="13" customWidth="1" min="87" max="87"/>
     <col width="13" customWidth="1" min="89" max="89"/>
-    <col width="13" customWidth="1" min="90" max="90"/>
     <col width="13" customWidth="1" min="91" max="91"/>
     <col width="13" customWidth="1" min="92" max="92"/>
     <col width="13" customWidth="1" min="93" max="93"/>
@@ -3859,25 +3859,25 @@
     <col width="13" customWidth="1" min="97" max="97"/>
     <col width="13" customWidth="1" min="98" max="98"/>
     <col width="13" customWidth="1" min="99" max="99"/>
+    <col width="13" customWidth="1" min="100" max="100"/>
     <col width="13" customWidth="1" min="101" max="101"/>
     <col width="13" customWidth="1" min="102" max="102"/>
-    <col width="13" customWidth="1" min="103" max="103"/>
     <col width="13" customWidth="1" min="104" max="104"/>
+    <col width="13" customWidth="1" min="105" max="105"/>
     <col width="13" customWidth="1" min="106" max="106"/>
     <col width="13" customWidth="1" min="107" max="107"/>
     <col width="13" customWidth="1" min="109" max="109"/>
     <col width="13" customWidth="1" min="110" max="110"/>
-    <col width="13" customWidth="1" min="111" max="111"/>
     <col width="13" customWidth="1" min="112" max="112"/>
     <col width="13" customWidth="1" min="113" max="113"/>
+    <col width="13" customWidth="1" min="114" max="114"/>
     <col width="13" customWidth="1" min="115" max="115"/>
     <col width="13" customWidth="1" min="116" max="116"/>
-    <col width="13" customWidth="1" min="117" max="117"/>
     <col width="13" customWidth="1" min="118" max="118"/>
+    <col width="13" customWidth="1" min="119" max="119"/>
     <col width="13" customWidth="1" min="120" max="120"/>
-    <col width="13" customWidth="1" min="122" max="122"/>
+    <col width="13" customWidth="1" min="121" max="121"/>
     <col width="13" customWidth="1" min="123" max="123"/>
-    <col width="13" customWidth="1" min="124" max="124"/>
     <col width="13" customWidth="1" min="125" max="125"/>
     <col width="13" customWidth="1" min="126" max="126"/>
     <col width="13" customWidth="1" min="127" max="127"/>
@@ -3893,10 +3893,16 @@
     <col width="13" customWidth="1" min="137" max="137"/>
     <col width="13" customWidth="1" min="138" max="138"/>
     <col width="13" customWidth="1" min="139" max="139"/>
+    <col width="13" customWidth="1" min="140" max="140"/>
     <col width="13" customWidth="1" min="141" max="141"/>
     <col width="13" customWidth="1" min="142" max="142"/>
     <col width="13" customWidth="1" min="143" max="143"/>
     <col width="13" customWidth="1" min="144" max="144"/>
+    <col width="13" customWidth="1" min="145" max="145"/>
+    <col width="13" customWidth="1" min="147" max="147"/>
+    <col width="13" customWidth="1" min="148" max="148"/>
+    <col width="13" customWidth="1" min="149" max="149"/>
+    <col width="13" customWidth="1" min="150" max="150"/>
   </cols>
   <sheetData>
     <row r="1" ht="29.25" customHeight="1">
@@ -4319,7 +4325,7 @@
       <c r="N17" s="85" t="n"/>
       <c r="O17" s="85" t="n"/>
     </row>
-    <row r="18" ht="150" customHeight="1">
+    <row r="18" ht="255" customHeight="1">
       <c r="A18" s="84" t="inlineStr">
         <is>
           <t>Estrategia</t>
@@ -4330,7 +4336,7 @@
       <c r="D18" s="85" t="n"/>
       <c r="E18" s="84" t="inlineStr">
         <is>
-          <t>Ventilador axial directo + rejillas de exfiltración</t>
+          <t>Ventilador axial mural Ø560 mm + cubierta intemperie con filtración + rejillas de exfiltración</t>
         </is>
       </c>
       <c r="F18" s="85" t="n"/>
@@ -4346,7 +4352,7 @@
       <c r="L18" s="85" t="n"/>
       <c r="M18" s="84" t="inlineStr">
         <is>
-          <t>Sin ductos de impulsión</t>
+          <t>Sin ductos de impulsión; montaje uniforme con la planta (REV2)</t>
         </is>
       </c>
       <c r="N18" s="85" t="n"/>
@@ -5799,13 +5805,13 @@
       <c r="L75" s="85" t="n"/>
       <c r="M75" s="84" t="inlineStr">
         <is>
-          <t>Para referencia</t>
+          <t>Para referencia (BC del CFD, histórica)</t>
         </is>
       </c>
       <c r="N75" s="85" t="n"/>
       <c r="O75" s="85" t="n"/>
     </row>
-    <row r="76" ht="75" customHeight="1">
+    <row r="76" ht="120" customHeight="1">
       <c r="A76" s="84" t="inlineStr">
         <is>
           <t>Radio del ventilador (CFD)</t>
@@ -5831,31 +5837,30 @@
       <c r="L76" s="85" t="n"/>
       <c r="M76" s="84" t="inlineStr">
         <is>
-          <t>Círculo de inyección</t>
+          <t>Círculo de inyección (BC del CFD, histórica)</t>
         </is>
       </c>
       <c r="N76" s="85" t="n"/>
       <c r="O76" s="85" t="n"/>
     </row>
-    <row r="77" ht="75" customHeight="1">
+    <row r="77" ht="165" customHeight="1">
       <c r="A77" s="84" t="inlineStr">
         <is>
-          <t>Velocidad de impulsión</t>
+          <t>Diámetro del impulsor seleccionado</t>
         </is>
       </c>
       <c r="B77" s="85" t="n"/>
       <c r="C77" s="85" t="n"/>
       <c r="D77" s="85" t="n"/>
-      <c r="E77" s="92">
-        <f>G32</f>
-        <v/>
+      <c r="E77" s="92" t="n">
+        <v>0.5600000000000001</v>
       </c>
       <c r="F77" s="93" t="n"/>
       <c r="G77" s="93" t="n"/>
       <c r="H77" s="93" t="n"/>
       <c r="I77" s="86" t="inlineStr">
         <is>
-          <t>m/s</t>
+          <t>m</t>
         </is>
       </c>
       <c r="J77" s="85" t="n"/>
@@ -5863,23 +5868,23 @@
       <c r="L77" s="85" t="n"/>
       <c r="M77" s="84" t="inlineStr">
         <is>
-          <t>Condición de entrada CFD</t>
+          <t>Ø560 mm — uniformidad con montaje típico de planta (REV2)</t>
         </is>
       </c>
       <c r="N77" s="85" t="n"/>
       <c r="O77" s="85" t="n"/>
     </row>
-    <row r="78" ht="105" customHeight="1">
+    <row r="78" ht="75" customHeight="1">
       <c r="A78" s="84" t="inlineStr">
         <is>
-          <t>Área neta total de rejillas de salida</t>
+          <t>Área de boca real (Ø560 mm)</t>
         </is>
       </c>
       <c r="B78" s="85" t="n"/>
       <c r="C78" s="85" t="n"/>
       <c r="D78" s="85" t="n"/>
       <c r="E78" s="92">
-        <f>J57</f>
+        <f>PI()*(0.56/2)^2</f>
         <v/>
       </c>
       <c r="F78" s="93" t="n"/>
@@ -5895,23 +5900,23 @@
       <c r="L78" s="85" t="n"/>
       <c r="M78" s="84" t="inlineStr">
         <is>
-          <t>A v=3 m/s</t>
+          <t>π × (D/2)²</t>
         </is>
       </c>
       <c r="N78" s="85" t="n"/>
       <c r="O78" s="85" t="n"/>
     </row>
-    <row r="79" ht="75" customHeight="1">
+    <row r="79" ht="90" customHeight="1">
       <c r="A79" s="84" t="inlineStr">
         <is>
-          <t>Número de rejillas de salida</t>
+          <t>Velocidad real en boca (Ø560 mm)</t>
         </is>
       </c>
       <c r="B79" s="85" t="n"/>
       <c r="C79" s="85" t="n"/>
       <c r="D79" s="85" t="n"/>
       <c r="E79" s="92">
-        <f>G34</f>
+        <f>J50/(PI()*(0.56/2)^2)</f>
         <v/>
       </c>
       <c r="F79" s="93" t="n"/>
@@ -5919,7 +5924,7 @@
       <c r="H79" s="93" t="n"/>
       <c r="I79" s="86" t="inlineStr">
         <is>
-          <t>unid.</t>
+          <t>m/s</t>
         </is>
       </c>
       <c r="J79" s="85" t="n"/>
@@ -5927,23 +5932,23 @@
       <c r="L79" s="85" t="n"/>
       <c r="M79" s="84" t="inlineStr">
         <is>
-          <t>Distribución propuesta</t>
+          <t>Q_s / A_boca real ≈ 4,33 m/s</t>
         </is>
       </c>
       <c r="N79" s="85" t="n"/>
       <c r="O79" s="85" t="n"/>
     </row>
-    <row r="80" ht="90" customHeight="1">
+    <row r="80" ht="75" customHeight="1">
       <c r="A80" s="84" t="inlineStr">
         <is>
-          <t>Área neta por rejilla de salida</t>
+          <t>Velocidad de impulsión</t>
         </is>
       </c>
       <c r="B80" s="85" t="n"/>
       <c r="C80" s="85" t="n"/>
       <c r="D80" s="85" t="n"/>
       <c r="E80" s="92">
-        <f>J58</f>
+        <f>G32</f>
         <v/>
       </c>
       <c r="F80" s="93" t="n"/>
@@ -5951,7 +5956,7 @@
       <c r="H80" s="93" t="n"/>
       <c r="I80" s="86" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m/s</t>
         </is>
       </c>
       <c r="J80" s="85" t="n"/>
@@ -5959,23 +5964,23 @@
       <c r="L80" s="85" t="n"/>
       <c r="M80" s="84" t="inlineStr">
         <is>
-          <t>Cada rejilla</t>
+          <t>Condición de entrada CFD</t>
         </is>
       </c>
       <c r="N80" s="85" t="n"/>
       <c r="O80" s="85" t="n"/>
     </row>
-    <row r="81" ht="75" customHeight="1">
+    <row r="81" ht="105" customHeight="1">
       <c r="A81" s="84" t="inlineStr">
         <is>
-          <t>Altura de rejilla de salida</t>
+          <t>Área neta total de rejillas de salida</t>
         </is>
       </c>
       <c r="B81" s="85" t="n"/>
       <c r="C81" s="85" t="n"/>
       <c r="D81" s="85" t="n"/>
       <c r="E81" s="92">
-        <f>J61</f>
+        <f>J57</f>
         <v/>
       </c>
       <c r="F81" s="93" t="n"/>
@@ -5983,7 +5988,7 @@
       <c r="H81" s="93" t="n"/>
       <c r="I81" s="86" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="J81" s="85" t="n"/>
@@ -5991,7 +5996,7 @@
       <c r="L81" s="85" t="n"/>
       <c r="M81" s="84" t="inlineStr">
         <is>
-          <t>Dimensiones para CFD</t>
+          <t>A v=3 m/s</t>
         </is>
       </c>
       <c r="N81" s="85" t="n"/>
@@ -6000,14 +6005,14 @@
     <row r="82" ht="75" customHeight="1">
       <c r="A82" s="84" t="inlineStr">
         <is>
-          <t>Ancho de rejilla de salida</t>
+          <t>Número de rejillas de salida</t>
         </is>
       </c>
       <c r="B82" s="85" t="n"/>
       <c r="C82" s="85" t="n"/>
       <c r="D82" s="85" t="n"/>
       <c r="E82" s="92">
-        <f>J62</f>
+        <f>G34</f>
         <v/>
       </c>
       <c r="F82" s="93" t="n"/>
@@ -6015,7 +6020,7 @@
       <c r="H82" s="93" t="n"/>
       <c r="I82" s="86" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>unid.</t>
         </is>
       </c>
       <c r="J82" s="85" t="n"/>
@@ -6023,23 +6028,23 @@
       <c r="L82" s="85" t="n"/>
       <c r="M82" s="84" t="inlineStr">
         <is>
-          <t>Dimensiones para CFD</t>
+          <t>Distribución propuesta</t>
         </is>
       </c>
       <c r="N82" s="85" t="n"/>
       <c r="O82" s="85" t="n"/>
     </row>
-    <row r="83" ht="120" customHeight="1">
+    <row r="83" ht="90" customHeight="1">
       <c r="A83" s="84" t="inlineStr">
         <is>
-          <t>Velocidad de exfiltración</t>
+          <t>Área neta por rejilla de salida</t>
         </is>
       </c>
       <c r="B83" s="85" t="n"/>
       <c r="C83" s="85" t="n"/>
       <c r="D83" s="85" t="n"/>
       <c r="E83" s="92">
-        <f>G33</f>
+        <f>J58</f>
         <v/>
       </c>
       <c r="F83" s="93" t="n"/>
@@ -6047,7 +6052,7 @@
       <c r="H83" s="93" t="n"/>
       <c r="I83" s="86" t="inlineStr">
         <is>
-          <t>m/s</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="J83" s="85" t="n"/>
@@ -6055,23 +6060,23 @@
       <c r="L83" s="85" t="n"/>
       <c r="M83" s="84" t="inlineStr">
         <is>
-          <t>Condición de salida CFD (pressure outlet)</t>
+          <t>Cada rejilla</t>
         </is>
       </c>
       <c r="N83" s="85" t="n"/>
       <c r="O83" s="85" t="n"/>
     </row>
-    <row r="84" ht="105" customHeight="1">
+    <row r="84" ht="75" customHeight="1">
       <c r="A84" s="84" t="inlineStr">
         <is>
-          <t>Pérdida de presión en rejillas</t>
+          <t>Altura de rejilla de salida</t>
         </is>
       </c>
       <c r="B84" s="85" t="n"/>
       <c r="C84" s="85" t="n"/>
       <c r="D84" s="85" t="n"/>
       <c r="E84" s="92">
-        <f>J63</f>
+        <f>J61</f>
         <v/>
       </c>
       <c r="F84" s="93" t="n"/>
@@ -6079,7 +6084,7 @@
       <c r="H84" s="93" t="n"/>
       <c r="I84" s="86" t="inlineStr">
         <is>
-          <t>Pa</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="J84" s="85" t="n"/>
@@ -6087,157 +6092,154 @@
       <c r="L84" s="85" t="n"/>
       <c r="M84" s="84" t="inlineStr">
         <is>
-          <t>Descarga libre a atmósfera, Cd=0.6</t>
+          <t>Dimensiones para CFD</t>
         </is>
       </c>
       <c r="N84" s="85" t="n"/>
       <c r="O84" s="85" t="n"/>
     </row>
-    <row r="85" ht="15" customHeight="1"/>
-    <row r="86" ht="135" customHeight="1">
-      <c r="A86" s="81" t="inlineStr">
+    <row r="85" ht="75" customHeight="1">
+      <c r="A85" s="84" t="inlineStr">
+        <is>
+          <t>Ancho de rejilla de salida</t>
+        </is>
+      </c>
+      <c r="B85" s="85" t="n"/>
+      <c r="C85" s="85" t="n"/>
+      <c r="D85" s="85" t="n"/>
+      <c r="E85" s="92">
+        <f>J62</f>
+        <v/>
+      </c>
+      <c r="F85" s="93" t="n"/>
+      <c r="G85" s="93" t="n"/>
+      <c r="H85" s="93" t="n"/>
+      <c r="I85" s="86" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="J85" s="85" t="n"/>
+      <c r="K85" s="85" t="n"/>
+      <c r="L85" s="85" t="n"/>
+      <c r="M85" s="84" t="inlineStr">
+        <is>
+          <t>Dimensiones para CFD</t>
+        </is>
+      </c>
+      <c r="N85" s="85" t="n"/>
+      <c r="O85" s="85" t="n"/>
+    </row>
+    <row r="86" ht="120" customHeight="1">
+      <c r="A86" s="84" t="inlineStr">
+        <is>
+          <t>Velocidad de exfiltración</t>
+        </is>
+      </c>
+      <c r="B86" s="85" t="n"/>
+      <c r="C86" s="85" t="n"/>
+      <c r="D86" s="85" t="n"/>
+      <c r="E86" s="92">
+        <f>G33</f>
+        <v/>
+      </c>
+      <c r="F86" s="93" t="n"/>
+      <c r="G86" s="93" t="n"/>
+      <c r="H86" s="93" t="n"/>
+      <c r="I86" s="86" t="inlineStr">
+        <is>
+          <t>m/s</t>
+        </is>
+      </c>
+      <c r="J86" s="85" t="n"/>
+      <c r="K86" s="85" t="n"/>
+      <c r="L86" s="85" t="n"/>
+      <c r="M86" s="84" t="inlineStr">
+        <is>
+          <t>Condición de salida CFD (pressure outlet)</t>
+        </is>
+      </c>
+      <c r="N86" s="85" t="n"/>
+      <c r="O86" s="85" t="n"/>
+    </row>
+    <row r="87" ht="105" customHeight="1">
+      <c r="A87" s="84" t="inlineStr">
+        <is>
+          <t>Pérdida de presión en rejillas</t>
+        </is>
+      </c>
+      <c r="B87" s="85" t="n"/>
+      <c r="C87" s="85" t="n"/>
+      <c r="D87" s="85" t="n"/>
+      <c r="E87" s="92">
+        <f>J63</f>
+        <v/>
+      </c>
+      <c r="F87" s="93" t="n"/>
+      <c r="G87" s="93" t="n"/>
+      <c r="H87" s="93" t="n"/>
+      <c r="I87" s="86" t="inlineStr">
+        <is>
+          <t>Pa</t>
+        </is>
+      </c>
+      <c r="J87" s="85" t="n"/>
+      <c r="K87" s="85" t="n"/>
+      <c r="L87" s="85" t="n"/>
+      <c r="M87" s="84" t="inlineStr">
+        <is>
+          <t>Descarga libre a atmósfera, Cd=0.6</t>
+        </is>
+      </c>
+      <c r="N87" s="85" t="n"/>
+      <c r="O87" s="85" t="n"/>
+    </row>
+    <row r="88" ht="15" customHeight="1"/>
+    <row r="89" ht="135" customHeight="1">
+      <c r="A89" s="81" t="inlineStr">
         <is>
           <t>5. SUSTENTACIÓN NORMATIVA — 12 RENOVACIONES/HORA</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="15" customHeight="1"/>
-    <row r="88" ht="60" customHeight="1">
-      <c r="A88" s="83" t="inlineStr">
+    <row r="90" ht="15" customHeight="1"/>
+    <row r="91" ht="60" customHeight="1">
+      <c r="A91" s="83" t="inlineStr">
         <is>
           <t>Norma / Guía</t>
         </is>
       </c>
-      <c r="B88" s="83" t="n"/>
-      <c r="C88" s="83" t="n"/>
-      <c r="D88" s="83" t="n"/>
-      <c r="E88" s="83" t="inlineStr">
+      <c r="B91" s="83" t="n"/>
+      <c r="C91" s="83" t="n"/>
+      <c r="D91" s="83" t="n"/>
+      <c r="E91" s="83" t="inlineStr">
         <is>
           <t>Año / Edición</t>
         </is>
       </c>
-      <c r="F88" s="83" t="n"/>
-      <c r="G88" s="83" t="n"/>
-      <c r="H88" s="83" t="n"/>
-      <c r="I88" s="83" t="inlineStr">
+      <c r="F91" s="83" t="n"/>
+      <c r="G91" s="83" t="n"/>
+      <c r="H91" s="83" t="n"/>
+      <c r="I91" s="83" t="inlineStr">
         <is>
           <t>Recomendación ACH</t>
         </is>
       </c>
-      <c r="J88" s="83" t="n"/>
-      <c r="K88" s="83" t="n"/>
-      <c r="L88" s="83" t="n"/>
-      <c r="M88" s="83" t="inlineStr">
+      <c r="J91" s="83" t="n"/>
+      <c r="K91" s="83" t="n"/>
+      <c r="L91" s="83" t="n"/>
+      <c r="M91" s="83" t="inlineStr">
         <is>
           <t>Observación</t>
         </is>
       </c>
-      <c r="N88" s="83" t="n"/>
-      <c r="O88" s="83" t="n"/>
-    </row>
-    <row r="89" ht="135" customHeight="1">
-      <c r="A89" s="84" t="inlineStr">
+      <c r="N91" s="83" t="n"/>
+      <c r="O91" s="83" t="n"/>
+    </row>
+    <row r="92" ht="135" customHeight="1">
+      <c r="A92" s="84" t="inlineStr">
         <is>
           <t>ASHRAE 170 — Ventilation of Health Care Facilities</t>
-        </is>
-      </c>
-      <c r="B89" s="85" t="n"/>
-      <c r="C89" s="85" t="n"/>
-      <c r="D89" s="85" t="n"/>
-      <c r="E89" s="86" t="inlineStr">
-        <is>
-          <t>2021</t>
-        </is>
-      </c>
-      <c r="F89" s="85" t="n"/>
-      <c r="G89" s="85" t="n"/>
-      <c r="H89" s="85" t="n"/>
-      <c r="I89" s="86" t="inlineStr">
-        <is>
-          <t>6–15 ACH</t>
-        </is>
-      </c>
-      <c r="J89" s="85" t="n"/>
-      <c r="K89" s="85" t="n"/>
-      <c r="L89" s="85" t="n"/>
-      <c r="M89" s="84" t="inlineStr">
-        <is>
-          <t>Laboratorios clínicos/procedimiento</t>
-        </is>
-      </c>
-      <c r="N89" s="85" t="n"/>
-      <c r="O89" s="85" t="n"/>
-    </row>
-    <row r="90" ht="120" customHeight="1">
-      <c r="A90" s="84" t="inlineStr">
-        <is>
-          <t>ASHRAE 62.1 — Ventilation for Acceptable IAQ</t>
-        </is>
-      </c>
-      <c r="B90" s="85" t="n"/>
-      <c r="C90" s="85" t="n"/>
-      <c r="D90" s="85" t="n"/>
-      <c r="E90" s="86" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="F90" s="85" t="n"/>
-      <c r="G90" s="85" t="n"/>
-      <c r="H90" s="85" t="n"/>
-      <c r="I90" s="86" t="inlineStr">
-        <is>
-          <t>Por ocupación y área</t>
-        </is>
-      </c>
-      <c r="J90" s="85" t="n"/>
-      <c r="K90" s="85" t="n"/>
-      <c r="L90" s="85" t="n"/>
-      <c r="M90" s="84" t="inlineStr">
-        <is>
-          <t>Caudal mínimo de aire exterior</t>
-        </is>
-      </c>
-      <c r="N90" s="85" t="n"/>
-      <c r="O90" s="85" t="n"/>
-    </row>
-    <row r="91" ht="120" customHeight="1">
-      <c r="A91" s="84" t="inlineStr">
-        <is>
-          <t>OSHA 29 CFR 1910.1450 — Laboratory Standard</t>
-        </is>
-      </c>
-      <c r="B91" s="85" t="n"/>
-      <c r="C91" s="85" t="n"/>
-      <c r="D91" s="85" t="n"/>
-      <c r="E91" s="86" t="inlineStr">
-        <is>
-          <t>2012</t>
-        </is>
-      </c>
-      <c r="F91" s="85" t="n"/>
-      <c r="G91" s="85" t="n"/>
-      <c r="H91" s="85" t="n"/>
-      <c r="I91" s="86" t="inlineStr">
-        <is>
-          <t>Según PEL</t>
-        </is>
-      </c>
-      <c r="J91" s="85" t="n"/>
-      <c r="K91" s="85" t="n"/>
-      <c r="L91" s="85" t="n"/>
-      <c r="M91" s="84" t="inlineStr">
-        <is>
-          <t>Ventilación para control de exposición</t>
-        </is>
-      </c>
-      <c r="N91" s="85" t="n"/>
-      <c r="O91" s="85" t="n"/>
-    </row>
-    <row r="92" ht="105" customHeight="1">
-      <c r="A92" s="84" t="inlineStr">
-        <is>
-          <t>NFPA 99 — Health Care Facilities Code</t>
         </is>
       </c>
       <c r="B92" s="85" t="n"/>
@@ -6253,7 +6255,7 @@
       <c r="H92" s="85" t="n"/>
       <c r="I92" s="86" t="inlineStr">
         <is>
-          <t>Cumplimiento de sistemas</t>
+          <t>6–15 ACH</t>
         </is>
       </c>
       <c r="J92" s="85" t="n"/>
@@ -6261,7 +6263,7 @@
       <c r="L92" s="85" t="n"/>
       <c r="M92" s="84" t="inlineStr">
         <is>
-          <t>Fiabilidad de sistemas de aire</t>
+          <t>Laboratorios clínicos/procedimiento</t>
         </is>
       </c>
       <c r="N92" s="85" t="n"/>
@@ -6270,7 +6272,7 @@
     <row r="93" ht="120" customHeight="1">
       <c r="A93" s="84" t="inlineStr">
         <is>
-          <t>WHO — Laboratory Biosafety Manual (BSL-2)</t>
+          <t>ASHRAE 62.1 — Ventilation for Acceptable IAQ</t>
         </is>
       </c>
       <c r="B93" s="85" t="n"/>
@@ -6278,7 +6280,7 @@
       <c r="D93" s="85" t="n"/>
       <c r="E93" s="86" t="inlineStr">
         <is>
-          <t>2004</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="F93" s="85" t="n"/>
@@ -6286,7 +6288,7 @@
       <c r="H93" s="85" t="n"/>
       <c r="I93" s="86" t="inlineStr">
         <is>
-          <t>6–12 ACH</t>
+          <t>Por ocupación y área</t>
         </is>
       </c>
       <c r="J93" s="85" t="n"/>
@@ -6294,7 +6296,7 @@
       <c r="L93" s="85" t="n"/>
       <c r="M93" s="84" t="inlineStr">
         <is>
-          <t>12 ACH = límite superior BSL-2</t>
+          <t>Caudal mínimo de aire exterior</t>
         </is>
       </c>
       <c r="N93" s="85" t="n"/>
@@ -6303,7 +6305,7 @@
     <row r="94" ht="120" customHeight="1">
       <c r="A94" s="84" t="inlineStr">
         <is>
-          <t>WHO — Laboratory Biosafety Manual (BSL-3)</t>
+          <t>OSHA 29 CFR 1910.1450 — Laboratory Standard</t>
         </is>
       </c>
       <c r="B94" s="85" t="n"/>
@@ -6311,7 +6313,7 @@
       <c r="D94" s="85" t="n"/>
       <c r="E94" s="86" t="inlineStr">
         <is>
-          <t>2004</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="F94" s="85" t="n"/>
@@ -6319,7 +6321,7 @@
       <c r="H94" s="85" t="n"/>
       <c r="I94" s="86" t="inlineStr">
         <is>
-          <t>12–15 ACH</t>
+          <t>Según PEL</t>
         </is>
       </c>
       <c r="J94" s="85" t="n"/>
@@ -6327,16 +6329,16 @@
       <c r="L94" s="85" t="n"/>
       <c r="M94" s="84" t="inlineStr">
         <is>
-          <t>12 ACH = umbral inferior BSL-3</t>
+          <t>Ventilación para control de exposición</t>
         </is>
       </c>
       <c r="N94" s="85" t="n"/>
       <c r="O94" s="85" t="n"/>
     </row>
-    <row r="95" ht="120" customHeight="1">
+    <row r="95" ht="105" customHeight="1">
       <c r="A95" s="84" t="inlineStr">
         <is>
-          <t>NIH — Design Requirements Manual</t>
+          <t>NFPA 99 — Health Care Facilities Code</t>
         </is>
       </c>
       <c r="B95" s="85" t="n"/>
@@ -6344,7 +6346,7 @@
       <c r="D95" s="85" t="n"/>
       <c r="E95" s="86" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F95" s="85" t="n"/>
@@ -6352,7 +6354,7 @@
       <c r="H95" s="85" t="n"/>
       <c r="I95" s="86" t="inlineStr">
         <is>
-          <t>10–12 ACH</t>
+          <t>Cumplimiento de sistemas</t>
         </is>
       </c>
       <c r="J95" s="85" t="n"/>
@@ -6360,7 +6362,7 @@
       <c r="L95" s="85" t="n"/>
       <c r="M95" s="84" t="inlineStr">
         <is>
-          <t>Punto de diseño para laboratorios biomédicos</t>
+          <t>Fiabilidad de sistemas de aire</t>
         </is>
       </c>
       <c r="N95" s="85" t="n"/>
@@ -6369,7 +6371,7 @@
     <row r="96" ht="120" customHeight="1">
       <c r="A96" s="84" t="inlineStr">
         <is>
-          <t>ASHRAE Handbook — Fundamentals</t>
+          <t>WHO — Laboratory Biosafety Manual (BSL-2)</t>
         </is>
       </c>
       <c r="B96" s="85" t="n"/>
@@ -6377,7 +6379,7 @@
       <c r="D96" s="85" t="n"/>
       <c r="E96" s="86" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2004</t>
         </is>
       </c>
       <c r="F96" s="85" t="n"/>
@@ -6385,7 +6387,7 @@
       <c r="H96" s="85" t="n"/>
       <c r="I96" s="86" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6–12 ACH</t>
         </is>
       </c>
       <c r="J96" s="85" t="n"/>
@@ -6393,7 +6395,7 @@
       <c r="L96" s="85" t="n"/>
       <c r="M96" s="84" t="inlineStr">
         <is>
-          <t>Coeficiente de descarga de orificios (Cd)</t>
+          <t>12 ACH = límite superior BSL-2</t>
         </is>
       </c>
       <c r="N96" s="85" t="n"/>
@@ -6402,7 +6404,7 @@
     <row r="97" ht="120" customHeight="1">
       <c r="A97" s="84" t="inlineStr">
         <is>
-          <t>RETIE (Colombia)</t>
+          <t>WHO — Laboratory Biosafety Manual (BSL-3)</t>
         </is>
       </c>
       <c r="B97" s="85" t="n"/>
@@ -6410,7 +6412,7 @@
       <c r="D97" s="85" t="n"/>
       <c r="E97" s="86" t="inlineStr">
         <is>
-          <t>vigente</t>
+          <t>2004</t>
         </is>
       </c>
       <c r="F97" s="85" t="n"/>
@@ -6418,7 +6420,7 @@
       <c r="H97" s="85" t="n"/>
       <c r="I97" s="86" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12–15 ACH</t>
         </is>
       </c>
       <c r="J97" s="85" t="n"/>
@@ -6426,16 +6428,16 @@
       <c r="L97" s="85" t="n"/>
       <c r="M97" s="84" t="inlineStr">
         <is>
-          <t>Seguridad eléctrica del motor del ventilador</t>
+          <t>12 ACH = umbral inferior BSL-3</t>
         </is>
       </c>
       <c r="N97" s="85" t="n"/>
       <c r="O97" s="85" t="n"/>
     </row>
-    <row r="98" ht="105" customHeight="1">
+    <row r="98" ht="120" customHeight="1">
       <c r="A98" s="84" t="inlineStr">
         <is>
-          <t>NTC 2050 (Colombia)</t>
+          <t>NIH — Design Requirements Manual</t>
         </is>
       </c>
       <c r="B98" s="85" t="n"/>
@@ -6443,7 +6445,7 @@
       <c r="D98" s="85" t="n"/>
       <c r="E98" s="86" t="inlineStr">
         <is>
-          <t>vigente</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="F98" s="85" t="n"/>
@@ -6451,7 +6453,7 @@
       <c r="H98" s="85" t="n"/>
       <c r="I98" s="86" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10–12 ACH</t>
         </is>
       </c>
       <c r="J98" s="85" t="n"/>
@@ -6459,16 +6461,16 @@
       <c r="L98" s="85" t="n"/>
       <c r="M98" s="84" t="inlineStr">
         <is>
-          <t>Circuitos y protecciones eléctricas</t>
+          <t>Punto de diseño para laboratorios biomédicos</t>
         </is>
       </c>
       <c r="N98" s="85" t="n"/>
       <c r="O98" s="85" t="n"/>
     </row>
-    <row r="99" ht="135" customHeight="1">
+    <row r="99" ht="120" customHeight="1">
       <c r="A99" s="84" t="inlineStr">
         <is>
-          <t>Resolución 0312/2019 MinSalud (Colombia)</t>
+          <t>ASHRAE Handbook — Fundamentals</t>
         </is>
       </c>
       <c r="B99" s="85" t="n"/>
@@ -6476,7 +6478,7 @@
       <c r="D99" s="85" t="n"/>
       <c r="E99" s="86" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F99" s="85" t="n"/>
@@ -6492,201 +6494,195 @@
       <c r="L99" s="85" t="n"/>
       <c r="M99" s="84" t="inlineStr">
         <is>
-          <t>Habilitación de servicios de salud (si aplica)</t>
+          <t>Coeficiente de descarga de orificios (Cd)</t>
         </is>
       </c>
       <c r="N99" s="85" t="n"/>
       <c r="O99" s="85" t="n"/>
     </row>
-    <row r="100" ht="15" customHeight="1"/>
-    <row r="101" ht="30" customHeight="1">
-      <c r="A101" s="82" t="inlineStr">
+    <row r="100" ht="120" customHeight="1">
+      <c r="A100" s="84" t="inlineStr">
+        <is>
+          <t>RETIE (Colombia)</t>
+        </is>
+      </c>
+      <c r="B100" s="85" t="n"/>
+      <c r="C100" s="85" t="n"/>
+      <c r="D100" s="85" t="n"/>
+      <c r="E100" s="86" t="inlineStr">
+        <is>
+          <t>vigente</t>
+        </is>
+      </c>
+      <c r="F100" s="85" t="n"/>
+      <c r="G100" s="85" t="n"/>
+      <c r="H100" s="85" t="n"/>
+      <c r="I100" s="86" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J100" s="85" t="n"/>
+      <c r="K100" s="85" t="n"/>
+      <c r="L100" s="85" t="n"/>
+      <c r="M100" s="84" t="inlineStr">
+        <is>
+          <t>Seguridad eléctrica del motor del ventilador</t>
+        </is>
+      </c>
+      <c r="N100" s="85" t="n"/>
+      <c r="O100" s="85" t="n"/>
+    </row>
+    <row r="101" ht="105" customHeight="1">
+      <c r="A101" s="84" t="inlineStr">
+        <is>
+          <t>NTC 2050 (Colombia)</t>
+        </is>
+      </c>
+      <c r="B101" s="85" t="n"/>
+      <c r="C101" s="85" t="n"/>
+      <c r="D101" s="85" t="n"/>
+      <c r="E101" s="86" t="inlineStr">
+        <is>
+          <t>vigente</t>
+        </is>
+      </c>
+      <c r="F101" s="85" t="n"/>
+      <c r="G101" s="85" t="n"/>
+      <c r="H101" s="85" t="n"/>
+      <c r="I101" s="86" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J101" s="85" t="n"/>
+      <c r="K101" s="85" t="n"/>
+      <c r="L101" s="85" t="n"/>
+      <c r="M101" s="84" t="inlineStr">
+        <is>
+          <t>Circuitos y protecciones eléctricas</t>
+        </is>
+      </c>
+      <c r="N101" s="85" t="n"/>
+      <c r="O101" s="85" t="n"/>
+    </row>
+    <row r="102" ht="135" customHeight="1">
+      <c r="A102" s="84" t="inlineStr">
+        <is>
+          <t>Resolución 0312/2019 MinSalud (Colombia)</t>
+        </is>
+      </c>
+      <c r="B102" s="85" t="n"/>
+      <c r="C102" s="85" t="n"/>
+      <c r="D102" s="85" t="n"/>
+      <c r="E102" s="86" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F102" s="85" t="n"/>
+      <c r="G102" s="85" t="n"/>
+      <c r="H102" s="85" t="n"/>
+      <c r="I102" s="86" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J102" s="85" t="n"/>
+      <c r="K102" s="85" t="n"/>
+      <c r="L102" s="85" t="n"/>
+      <c r="M102" s="84" t="inlineStr">
+        <is>
+          <t>Habilitación de servicios de salud (si aplica)</t>
+        </is>
+      </c>
+      <c r="N102" s="85" t="n"/>
+      <c r="O102" s="85" t="n"/>
+    </row>
+    <row r="103" ht="15" customHeight="1"/>
+    <row r="104" ht="30" customHeight="1">
+      <c r="A104" s="82" t="inlineStr">
         <is>
           <t>Conclusión</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="375" customHeight="1">
-      <c r="A102" s="87" t="inlineStr">
+    <row r="105" ht="375" customHeight="1">
+      <c r="A105" s="87" t="inlineStr">
         <is>
           <t>La selección de 12 renovaciones de aire por hora está sustentada por las guías internacionales de bioseguridad (WHO BSL-2/BSL-3, NIH DRM) y los estándares de ventilación de ASHRAE para instalaciones de salud. El marco regulatorio local (RETIE, NTC 2050, Resolución 0312/2019) aplica a la infraestructura y seguridad eléctrica del equipo; no existe norma colombiana que fije un valor de ACH distinto para este caso.</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="15" customHeight="1"/>
-    <row r="104" ht="15" customHeight="1"/>
-    <row r="105" ht="15" customHeight="1"/>
-    <row r="106" ht="135" customHeight="1">
-      <c r="A106" s="81" t="inlineStr">
+    <row r="106" ht="15" customHeight="1"/>
+    <row r="107" ht="15" customHeight="1"/>
+    <row r="108" ht="15" customHeight="1"/>
+    <row r="109" ht="135" customHeight="1">
+      <c r="A109" s="81" t="inlineStr">
         <is>
           <t>6. ESCENARIOS DE FILTRACIÓN Y MOTOR RECOMENDADO</t>
         </is>
       </c>
     </row>
-    <row r="107" ht="600" customHeight="1">
-      <c r="A107" s="87" t="inlineStr">
+    <row r="110" ht="600" customHeight="1">
+      <c r="A110" s="87" t="inlineStr">
         <is>
           <t>ΔP_vent total = ΔP_filtro + ΔP_rejillas (11 Pa). Sin presurización (REV1: cambio de alcance del cliente). El caudal Q_s se toma del paso 4 de la sección 3 (celda J50). Sitio: Cajicá, Cundinamarca (2 558 msnm, ρ = 0.88 kg/m³).</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="15" customHeight="1"/>
-    <row r="109" ht="75" customHeight="1">
-      <c r="A109" s="83" t="inlineStr">
+    <row r="111" ht="15" customHeight="1"/>
+    <row r="112" ht="75" customHeight="1">
+      <c r="A112" s="83" t="inlineStr">
         <is>
           <t>Escenario de filtración</t>
         </is>
       </c>
-      <c r="B109" s="83" t="n"/>
-      <c r="C109" s="83" t="n"/>
-      <c r="D109" s="83" t="inlineStr">
+      <c r="B112" s="83" t="n"/>
+      <c r="C112" s="83" t="n"/>
+      <c r="D112" s="83" t="inlineStr">
         <is>
           <t>ΔP filtro (Pa)</t>
         </is>
       </c>
-      <c r="E109" s="83" t="n"/>
-      <c r="F109" s="83" t="n"/>
-      <c r="G109" s="83" t="inlineStr">
+      <c r="E112" s="83" t="n"/>
+      <c r="F112" s="83" t="n"/>
+      <c r="G112" s="83" t="inlineStr">
         <is>
           <t>ΔP vent total (Pa)</t>
         </is>
       </c>
-      <c r="H109" s="83" t="n"/>
-      <c r="I109" s="83" t="n"/>
-      <c r="J109" s="83" t="inlineStr">
+      <c r="H112" s="83" t="n"/>
+      <c r="I112" s="83" t="n"/>
+      <c r="J112" s="83" t="inlineStr">
         <is>
           <t>P teórica (kW)</t>
         </is>
       </c>
-      <c r="K109" s="83" t="n"/>
-      <c r="L109" s="83" t="inlineStr">
+      <c r="K112" s="83" t="n"/>
+      <c r="L112" s="83" t="inlineStr">
         <is>
           <t>P teórica (HP)</t>
         </is>
       </c>
-      <c r="M109" s="83" t="n"/>
-      <c r="N109" s="83" t="inlineStr">
+      <c r="M112" s="83" t="n"/>
+      <c r="N112" s="83" t="inlineStr">
         <is>
           <t>Motor recomendado (HP)</t>
         </is>
       </c>
-      <c r="O109" s="83" t="n"/>
-    </row>
-    <row r="110" ht="75" customHeight="1">
-      <c r="A110" s="84" t="inlineStr">
+      <c r="O112" s="83" t="n"/>
+    </row>
+    <row r="113" ht="75" customHeight="1">
+      <c r="A113" s="84" t="inlineStr">
         <is>
           <t>MERV 13-14 limpio</t>
-        </is>
-      </c>
-      <c r="B110" s="85" t="n"/>
-      <c r="C110" s="85" t="n"/>
-      <c r="D110" s="94" t="n">
-        <v>59</v>
-      </c>
-      <c r="E110" s="95" t="n"/>
-      <c r="F110" s="95" t="n"/>
-      <c r="G110" s="94">
-        <f>D110+11</f>
-        <v/>
-      </c>
-      <c r="H110" s="95" t="n"/>
-      <c r="I110" s="95" t="n"/>
-      <c r="J110" s="96">
-        <f>J50*G110/(0.55*1000)</f>
-        <v/>
-      </c>
-      <c r="K110" s="97" t="n"/>
-      <c r="L110" s="96">
-        <f>J110*1.341</f>
-        <v/>
-      </c>
-      <c r="M110" s="97" t="n"/>
-      <c r="N110" s="94">
-        <f>CEILING(L110*1.5,0.25)</f>
-        <v/>
-      </c>
-      <c r="O110" s="95" t="n"/>
-    </row>
-    <row r="111" ht="75" customHeight="1">
-      <c r="A111" s="84" t="inlineStr">
-        <is>
-          <t>MERV 13-14 cargado (diseño)</t>
-        </is>
-      </c>
-      <c r="B111" s="85" t="n"/>
-      <c r="C111" s="85" t="n"/>
-      <c r="D111" s="94" t="n">
-        <v>154</v>
-      </c>
-      <c r="E111" s="95" t="n"/>
-      <c r="F111" s="95" t="n"/>
-      <c r="G111" s="94">
-        <f>D111+11</f>
-        <v/>
-      </c>
-      <c r="H111" s="95" t="n"/>
-      <c r="I111" s="95" t="n"/>
-      <c r="J111" s="96">
-        <f>J50*G111/(0.55*1000)</f>
-        <v/>
-      </c>
-      <c r="K111" s="97" t="n"/>
-      <c r="L111" s="96">
-        <f>J111*1.341</f>
-        <v/>
-      </c>
-      <c r="M111" s="97" t="n"/>
-      <c r="N111" s="94">
-        <f>CEILING(L111*1.5,0.25)</f>
-        <v/>
-      </c>
-      <c r="O111" s="95" t="n"/>
-    </row>
-    <row r="112" ht="135" customHeight="1">
-      <c r="A112" s="84" t="inlineStr">
-        <is>
-          <t>HEPA H13 limpio (referencia histórica — no aplica)</t>
-        </is>
-      </c>
-      <c r="B112" s="85" t="n"/>
-      <c r="C112" s="85" t="n"/>
-      <c r="D112" s="94" t="n">
-        <v>250</v>
-      </c>
-      <c r="E112" s="95" t="n"/>
-      <c r="F112" s="95" t="n"/>
-      <c r="G112" s="94">
-        <f>D112+11</f>
-        <v/>
-      </c>
-      <c r="H112" s="95" t="n"/>
-      <c r="I112" s="95" t="n"/>
-      <c r="J112" s="96">
-        <f>J50*G112/(0.55*1000)</f>
-        <v/>
-      </c>
-      <c r="K112" s="97" t="n"/>
-      <c r="L112" s="96">
-        <f>J112*1.341</f>
-        <v/>
-      </c>
-      <c r="M112" s="97" t="n"/>
-      <c r="N112" s="94">
-        <f>CEILING(L112*1.5,0.25)</f>
-        <v/>
-      </c>
-      <c r="O112" s="95" t="n"/>
-    </row>
-    <row r="113" ht="150" customHeight="1">
-      <c r="A113" s="84" t="inlineStr">
-        <is>
-          <t>HEPA H13 cargado (referencia histórica — no aplica)</t>
         </is>
       </c>
       <c r="B113" s="85" t="n"/>
       <c r="C113" s="85" t="n"/>
       <c r="D113" s="94" t="n">
-        <v>600</v>
+        <v>59</v>
       </c>
       <c r="E113" s="95" t="n"/>
       <c r="F113" s="95" t="n"/>
@@ -6712,172 +6708,181 @@
       </c>
       <c r="O113" s="95" t="n"/>
     </row>
-    <row r="114" ht="15" customHeight="1"/>
-    <row r="115" ht="15" customHeight="1">
-      <c r="A115" s="82" t="inlineStr">
+    <row r="114" ht="75" customHeight="1">
+      <c r="A114" s="84" t="inlineStr">
+        <is>
+          <t>MERV 13-14 cargado (diseño)</t>
+        </is>
+      </c>
+      <c r="B114" s="85" t="n"/>
+      <c r="C114" s="85" t="n"/>
+      <c r="D114" s="94" t="n">
+        <v>154</v>
+      </c>
+      <c r="E114" s="95" t="n"/>
+      <c r="F114" s="95" t="n"/>
+      <c r="G114" s="94">
+        <f>D114+11</f>
+        <v/>
+      </c>
+      <c r="H114" s="95" t="n"/>
+      <c r="I114" s="95" t="n"/>
+      <c r="J114" s="96">
+        <f>J50*G114/(0.55*1000)</f>
+        <v/>
+      </c>
+      <c r="K114" s="97" t="n"/>
+      <c r="L114" s="96">
+        <f>J114*1.341</f>
+        <v/>
+      </c>
+      <c r="M114" s="97" t="n"/>
+      <c r="N114" s="94">
+        <f>CEILING(L114*1.5,0.25)</f>
+        <v/>
+      </c>
+      <c r="O114" s="95" t="n"/>
+    </row>
+    <row r="115" ht="135" customHeight="1">
+      <c r="A115" s="84" t="inlineStr">
+        <is>
+          <t>HEPA H13 limpio (referencia histórica — no aplica)</t>
+        </is>
+      </c>
+      <c r="B115" s="85" t="n"/>
+      <c r="C115" s="85" t="n"/>
+      <c r="D115" s="94" t="n">
+        <v>250</v>
+      </c>
+      <c r="E115" s="95" t="n"/>
+      <c r="F115" s="95" t="n"/>
+      <c r="G115" s="94">
+        <f>D115+11</f>
+        <v/>
+      </c>
+      <c r="H115" s="95" t="n"/>
+      <c r="I115" s="95" t="n"/>
+      <c r="J115" s="96">
+        <f>J50*G115/(0.55*1000)</f>
+        <v/>
+      </c>
+      <c r="K115" s="97" t="n"/>
+      <c r="L115" s="96">
+        <f>J115*1.341</f>
+        <v/>
+      </c>
+      <c r="M115" s="97" t="n"/>
+      <c r="N115" s="94">
+        <f>CEILING(L115*1.5,0.25)</f>
+        <v/>
+      </c>
+      <c r="O115" s="95" t="n"/>
+    </row>
+    <row r="116" ht="150" customHeight="1">
+      <c r="A116" s="84" t="inlineStr">
+        <is>
+          <t>HEPA H13 cargado (referencia histórica — no aplica)</t>
+        </is>
+      </c>
+      <c r="B116" s="85" t="n"/>
+      <c r="C116" s="85" t="n"/>
+      <c r="D116" s="94" t="n">
+        <v>600</v>
+      </c>
+      <c r="E116" s="95" t="n"/>
+      <c r="F116" s="95" t="n"/>
+      <c r="G116" s="94">
+        <f>D116+11</f>
+        <v/>
+      </c>
+      <c r="H116" s="95" t="n"/>
+      <c r="I116" s="95" t="n"/>
+      <c r="J116" s="96">
+        <f>J50*G116/(0.55*1000)</f>
+        <v/>
+      </c>
+      <c r="K116" s="97" t="n"/>
+      <c r="L116" s="96">
+        <f>J116*1.341</f>
+        <v/>
+      </c>
+      <c r="M116" s="97" t="n"/>
+      <c r="N116" s="94">
+        <f>CEILING(L116*1.5,0.25)</f>
+        <v/>
+      </c>
+      <c r="O116" s="95" t="n"/>
+    </row>
+    <row r="117" ht="15" customHeight="1"/>
+    <row r="118" ht="15" customHeight="1">
+      <c r="A118" s="82" t="inlineStr">
         <is>
           <t>Nota:</t>
         </is>
       </c>
     </row>
-    <row r="116" ht="525" customHeight="1">
-      <c r="A116" s="87" t="inlineStr">
-        <is>
-          <t>El motor provisional de 0.75 HP TEFC anticorrosivo corresponde al escenario MERV 13-14 cargado (punto de diseño), con margen de servicio 1.5 sobre la potencia teórica; la potencia definitiva se fija con la curva del ventilador axial seleccionado. Los escenarios HEPA son solo referencia histórica: el laboratorio de análisis industrial NO requiere HEPA. Para selección de ventilador en catálogo (ρ = 1.2 kg/m³), usar el punto equivalente 3 840 m³/h @ 225 Pa (diseño) o 95 Pa (limpio). La potencia se recalcula automáticamente si cambia el caudal en la sección 3. DESARROLLO DE CÁLCULOS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="117" ht="15" customHeight="1"/>
-    <row r="118" ht="15" customHeight="1"/>
-    <row r="119" ht="15" customHeight="1"/>
-    <row r="120" ht="120" customHeight="1">
-      <c r="A120" s="81" t="inlineStr">
+    <row r="119" ht="645" customHeight="1">
+      <c r="A119" s="87" t="inlineStr">
+        <is>
+          <t>El motor provisional de 0.75 HP TEFC encapsulado anticorrosivo (en la corriente de aire, transmisión directa del ventilador mural Ø560 mm — uniformidad con el montaje típico de planta, REV2) corresponde al escenario MERV 13-14 cargado (punto de diseño), con margen de servicio 1.5 sobre la potencia teórica; la potencia definitiva se fija con la curva del ventilador axial seleccionado. Los escenarios HEPA son solo referencia histórica: el laboratorio de análisis industrial NO requiere HEPA. Para selección de ventilador en catálogo (ρ = 1.2 kg/m³), usar el punto equivalente 3 840 m³/h @ 225 Pa (diseño) o 95 Pa (limpio). La potencia se recalcula automáticamente si cambia el caudal en la sección 3. DESARROLLO DE CÁLCULOS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="15" customHeight="1"/>
+    <row r="121" ht="15" customHeight="1"/>
+    <row r="122" ht="15" customHeight="1"/>
+    <row r="123" ht="120" customHeight="1">
+      <c r="A123" s="81" t="inlineStr">
         <is>
           <t>7. VISTA RÁPIDA — RESULTADOS (FÓRMULAS VIVAS)</t>
         </is>
       </c>
     </row>
-    <row r="121" ht="15" customHeight="1"/>
-    <row r="122" ht="30" customHeight="1">
-      <c r="A122" s="83" t="inlineStr">
+    <row r="124" ht="15" customHeight="1"/>
+    <row r="125" ht="30" customHeight="1">
+      <c r="A125" s="83" t="inlineStr">
         <is>
           <t>Parámetro</t>
         </is>
       </c>
-      <c r="B122" s="83" t="n"/>
-      <c r="C122" s="83" t="n"/>
-      <c r="D122" s="83" t="n"/>
-      <c r="E122" s="83" t="inlineStr">
+      <c r="B125" s="83" t="n"/>
+      <c r="C125" s="83" t="n"/>
+      <c r="D125" s="83" t="n"/>
+      <c r="E125" s="83" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="F122" s="83" t="n"/>
-      <c r="G122" s="83" t="n"/>
-      <c r="H122" s="83" t="n"/>
-      <c r="I122" s="83" t="inlineStr">
+      <c r="F125" s="83" t="n"/>
+      <c r="G125" s="83" t="n"/>
+      <c r="H125" s="83" t="n"/>
+      <c r="I125" s="83" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="J122" s="83" t="n"/>
-      <c r="K122" s="83" t="n"/>
-      <c r="L122" s="83" t="n"/>
-      <c r="M122" s="83" t="inlineStr">
+      <c r="J125" s="83" t="n"/>
+      <c r="K125" s="83" t="n"/>
+      <c r="L125" s="83" t="n"/>
+      <c r="M125" s="83" t="inlineStr">
         <is>
           <t>Observación</t>
         </is>
       </c>
-      <c r="N122" s="83" t="n"/>
-      <c r="O122" s="83" t="n"/>
-    </row>
-    <row r="123" ht="90" customHeight="1">
-      <c r="A123" s="84" t="inlineStr">
+      <c r="N125" s="83" t="n"/>
+      <c r="O125" s="83" t="n"/>
+    </row>
+    <row r="126" ht="90" customHeight="1">
+      <c r="A126" s="84" t="inlineStr">
         <is>
           <t>Caudal de diseño</t>
-        </is>
-      </c>
-      <c r="B123" s="85" t="n"/>
-      <c r="C123" s="85" t="n"/>
-      <c r="D123" s="85" t="n"/>
-      <c r="E123" s="92">
-        <f>J47</f>
-        <v/>
-      </c>
-      <c r="F123" s="93" t="n"/>
-      <c r="G123" s="93" t="n"/>
-      <c r="H123" s="93" t="n"/>
-      <c r="I123" s="86" t="inlineStr">
-        <is>
-          <t>m³/min</t>
-        </is>
-      </c>
-      <c r="J123" s="85" t="n"/>
-      <c r="K123" s="85" t="n"/>
-      <c r="L123" s="85" t="n"/>
-      <c r="M123" s="84" t="inlineStr">
-        <is>
-          <t>Caudal de impulsión requerido</t>
-        </is>
-      </c>
-      <c r="N123" s="85" t="n"/>
-      <c r="O123" s="85" t="n"/>
-    </row>
-    <row r="124" ht="105" customHeight="1">
-      <c r="A124" s="84" t="inlineStr">
-        <is>
-          <t>Caudal de diseño</t>
-        </is>
-      </c>
-      <c r="B124" s="85" t="n"/>
-      <c r="C124" s="85" t="n"/>
-      <c r="D124" s="85" t="n"/>
-      <c r="E124" s="92">
-        <f>J48</f>
-        <v/>
-      </c>
-      <c r="F124" s="93" t="n"/>
-      <c r="G124" s="93" t="n"/>
-      <c r="H124" s="93" t="n"/>
-      <c r="I124" s="86" t="inlineStr">
-        <is>
-          <t>m³/h</t>
-        </is>
-      </c>
-      <c r="J124" s="85" t="n"/>
-      <c r="K124" s="85" t="n"/>
-      <c r="L124" s="85" t="n"/>
-      <c r="M124" s="84" t="inlineStr">
-        <is>
-          <t>Equivalente en metros cúbicos por hora</t>
-        </is>
-      </c>
-      <c r="N124" s="85" t="n"/>
-      <c r="O124" s="85" t="n"/>
-    </row>
-    <row r="125" ht="105" customHeight="1">
-      <c r="A125" s="84" t="inlineStr">
-        <is>
-          <t>Caudal de diseño</t>
-        </is>
-      </c>
-      <c r="B125" s="85" t="n"/>
-      <c r="C125" s="85" t="n"/>
-      <c r="D125" s="85" t="n"/>
-      <c r="E125" s="92">
-        <f>J49</f>
-        <v/>
-      </c>
-      <c r="F125" s="93" t="n"/>
-      <c r="G125" s="93" t="n"/>
-      <c r="H125" s="93" t="n"/>
-      <c r="I125" s="86" t="inlineStr">
-        <is>
-          <t>CFM</t>
-        </is>
-      </c>
-      <c r="J125" s="85" t="n"/>
-      <c r="K125" s="85" t="n"/>
-      <c r="L125" s="85" t="n"/>
-      <c r="M125" s="84" t="inlineStr">
-        <is>
-          <t>Equivalente en pies cúbicos por minuto</t>
-        </is>
-      </c>
-      <c r="N125" s="85" t="n"/>
-      <c r="O125" s="85" t="n"/>
-    </row>
-    <row r="126" ht="105" customHeight="1">
-      <c r="A126" s="84" t="inlineStr">
-        <is>
-          <t>Potencia teórica del ventilador</t>
         </is>
       </c>
       <c r="B126" s="85" t="n"/>
       <c r="C126" s="85" t="n"/>
       <c r="D126" s="85" t="n"/>
       <c r="E126" s="92">
-        <f>J51</f>
+        <f>J47</f>
         <v/>
       </c>
       <c r="F126" s="93" t="n"/>
@@ -6885,7 +6890,7 @@
       <c r="H126" s="93" t="n"/>
       <c r="I126" s="86" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>m³/min</t>
         </is>
       </c>
       <c r="J126" s="85" t="n"/>
@@ -6893,23 +6898,23 @@
       <c r="L126" s="85" t="n"/>
       <c r="M126" s="84" t="inlineStr">
         <is>
-          <t>Escenario MERV cargado a 165 Pa (axial)</t>
+          <t>Caudal de impulsión requerido</t>
         </is>
       </c>
       <c r="N126" s="85" t="n"/>
       <c r="O126" s="85" t="n"/>
     </row>
-    <row r="127" ht="90" customHeight="1">
+    <row r="127" ht="105" customHeight="1">
       <c r="A127" s="84" t="inlineStr">
         <is>
-          <t>Potencia teórica del ventilador</t>
+          <t>Caudal de diseño</t>
         </is>
       </c>
       <c r="B127" s="85" t="n"/>
       <c r="C127" s="85" t="n"/>
       <c r="D127" s="85" t="n"/>
       <c r="E127" s="92">
-        <f>J52</f>
+        <f>J48</f>
         <v/>
       </c>
       <c r="F127" s="93" t="n"/>
@@ -6917,7 +6922,7 @@
       <c r="H127" s="93" t="n"/>
       <c r="I127" s="86" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>m³/h</t>
         </is>
       </c>
       <c r="J127" s="85" t="n"/>
@@ -6925,7 +6930,7 @@
       <c r="L127" s="85" t="n"/>
       <c r="M127" s="84" t="inlineStr">
         <is>
-          <t>Unidades imperiales</t>
+          <t>Equivalente en metros cúbicos por hora</t>
         </is>
       </c>
       <c r="N127" s="85" t="n"/>
@@ -6934,14 +6939,14 @@
     <row r="128" ht="105" customHeight="1">
       <c r="A128" s="84" t="inlineStr">
         <is>
-          <t>Potencia instalada recomendada</t>
+          <t>Caudal de diseño</t>
         </is>
       </c>
       <c r="B128" s="85" t="n"/>
       <c r="C128" s="85" t="n"/>
       <c r="D128" s="85" t="n"/>
       <c r="E128" s="92">
-        <f>CEILING(J52*1.5,0.25)</f>
+        <f>J49</f>
         <v/>
       </c>
       <c r="F128" s="93" t="n"/>
@@ -6949,7 +6954,7 @@
       <c r="H128" s="93" t="n"/>
       <c r="I128" s="86" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>CFM</t>
         </is>
       </c>
       <c r="J128" s="85" t="n"/>
@@ -6957,23 +6962,23 @@
       <c r="L128" s="85" t="n"/>
       <c r="M128" s="84" t="inlineStr">
         <is>
-          <t>×1.5 margen de servicio (provisional)</t>
+          <t>Equivalente en pies cúbicos por minuto</t>
         </is>
       </c>
       <c r="N128" s="85" t="n"/>
       <c r="O128" s="85" t="n"/>
     </row>
-    <row r="129" ht="90" customHeight="1">
+    <row r="129" ht="105" customHeight="1">
       <c r="A129" s="84" t="inlineStr">
         <is>
-          <t>Área de impulsión del ventilador</t>
+          <t>Potencia teórica del ventilador</t>
         </is>
       </c>
       <c r="B129" s="85" t="n"/>
       <c r="C129" s="85" t="n"/>
       <c r="D129" s="85" t="n"/>
       <c r="E129" s="92">
-        <f>J53</f>
+        <f>J51</f>
         <v/>
       </c>
       <c r="F129" s="93" t="n"/>
@@ -6981,7 +6986,7 @@
       <c r="H129" s="93" t="n"/>
       <c r="I129" s="86" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="J129" s="85" t="n"/>
@@ -6989,23 +6994,23 @@
       <c r="L129" s="85" t="n"/>
       <c r="M129" s="84" t="inlineStr">
         <is>
-          <t>Boca del ventilador</t>
+          <t>Escenario MERV cargado a 165 Pa (axial)</t>
         </is>
       </c>
       <c r="N129" s="85" t="n"/>
       <c r="O129" s="85" t="n"/>
     </row>
-    <row r="130" ht="105" customHeight="1">
+    <row r="130" ht="90" customHeight="1">
       <c r="A130" s="84" t="inlineStr">
         <is>
-          <t>Diámetro equivalente del ventilador</t>
+          <t>Potencia teórica del ventilador</t>
         </is>
       </c>
       <c r="B130" s="85" t="n"/>
       <c r="C130" s="85" t="n"/>
       <c r="D130" s="85" t="n"/>
       <c r="E130" s="92">
-        <f>J54</f>
+        <f>J52</f>
         <v/>
       </c>
       <c r="F130" s="93" t="n"/>
@@ -7013,7 +7018,7 @@
       <c r="H130" s="93" t="n"/>
       <c r="I130" s="86" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="J130" s="85" t="n"/>
@@ -7021,23 +7026,23 @@
       <c r="L130" s="85" t="n"/>
       <c r="M130" s="84" t="inlineStr">
         <is>
-          <t>Para referencia</t>
+          <t>Unidades imperiales</t>
         </is>
       </c>
       <c r="N130" s="85" t="n"/>
       <c r="O130" s="85" t="n"/>
     </row>
-    <row r="131" ht="75" customHeight="1">
+    <row r="131" ht="105" customHeight="1">
       <c r="A131" s="84" t="inlineStr">
         <is>
-          <t>Radio del ventilador (CFD)</t>
+          <t>Potencia instalada recomendada</t>
         </is>
       </c>
       <c r="B131" s="85" t="n"/>
       <c r="C131" s="85" t="n"/>
       <c r="D131" s="85" t="n"/>
       <c r="E131" s="92">
-        <f>J56</f>
+        <f>CEILING(J52*1.5,0.25)</f>
         <v/>
       </c>
       <c r="F131" s="93" t="n"/>
@@ -7045,7 +7050,7 @@
       <c r="H131" s="93" t="n"/>
       <c r="I131" s="86" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="J131" s="85" t="n"/>
@@ -7053,23 +7058,23 @@
       <c r="L131" s="85" t="n"/>
       <c r="M131" s="84" t="inlineStr">
         <is>
-          <t>Círculo de inyección</t>
+          <t>×1.5 margen de servicio (provisional)</t>
         </is>
       </c>
       <c r="N131" s="85" t="n"/>
       <c r="O131" s="85" t="n"/>
     </row>
-    <row r="132" ht="75" customHeight="1">
+    <row r="132" ht="90" customHeight="1">
       <c r="A132" s="84" t="inlineStr">
         <is>
-          <t>Velocidad de impulsión</t>
+          <t>Área de impulsión del ventilador</t>
         </is>
       </c>
       <c r="B132" s="85" t="n"/>
       <c r="C132" s="85" t="n"/>
       <c r="D132" s="85" t="n"/>
       <c r="E132" s="92">
-        <f>G32</f>
+        <f>J53</f>
         <v/>
       </c>
       <c r="F132" s="93" t="n"/>
@@ -7077,7 +7082,7 @@
       <c r="H132" s="93" t="n"/>
       <c r="I132" s="86" t="inlineStr">
         <is>
-          <t>m/s</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="J132" s="85" t="n"/>
@@ -7085,7 +7090,7 @@
       <c r="L132" s="85" t="n"/>
       <c r="M132" s="84" t="inlineStr">
         <is>
-          <t>Condición de entrada CFD</t>
+          <t>Boca del ventilador</t>
         </is>
       </c>
       <c r="N132" s="85" t="n"/>
@@ -7094,14 +7099,14 @@
     <row r="133" ht="105" customHeight="1">
       <c r="A133" s="84" t="inlineStr">
         <is>
-          <t>Área neta total de rejillas de salida</t>
+          <t>Diámetro equivalente del ventilador</t>
         </is>
       </c>
       <c r="B133" s="85" t="n"/>
       <c r="C133" s="85" t="n"/>
       <c r="D133" s="85" t="n"/>
       <c r="E133" s="92">
-        <f>J57</f>
+        <f>J54</f>
         <v/>
       </c>
       <c r="F133" s="93" t="n"/>
@@ -7109,7 +7114,7 @@
       <c r="H133" s="93" t="n"/>
       <c r="I133" s="86" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
       <c r="J133" s="85" t="n"/>
@@ -7117,23 +7122,23 @@
       <c r="L133" s="85" t="n"/>
       <c r="M133" s="84" t="inlineStr">
         <is>
-          <t>A v=3 m/s</t>
+          <t>Para referencia (BC del CFD, histórica)</t>
         </is>
       </c>
       <c r="N133" s="85" t="n"/>
       <c r="O133" s="85" t="n"/>
     </row>
-    <row r="134" ht="75" customHeight="1">
+    <row r="134" ht="120" customHeight="1">
       <c r="A134" s="84" t="inlineStr">
         <is>
-          <t>Número de rejillas de salida</t>
+          <t>Radio del ventilador (CFD)</t>
         </is>
       </c>
       <c r="B134" s="85" t="n"/>
       <c r="C134" s="85" t="n"/>
       <c r="D134" s="85" t="n"/>
       <c r="E134" s="92">
-        <f>G34</f>
+        <f>J56</f>
         <v/>
       </c>
       <c r="F134" s="93" t="n"/>
@@ -7141,7 +7146,7 @@
       <c r="H134" s="93" t="n"/>
       <c r="I134" s="86" t="inlineStr">
         <is>
-          <t>unid.</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="J134" s="85" t="n"/>
@@ -7149,31 +7154,30 @@
       <c r="L134" s="85" t="n"/>
       <c r="M134" s="84" t="inlineStr">
         <is>
-          <t>Distribución propuesta</t>
+          <t>Círculo de inyección (BC del CFD, histórica)</t>
         </is>
       </c>
       <c r="N134" s="85" t="n"/>
       <c r="O134" s="85" t="n"/>
     </row>
-    <row r="135" ht="90" customHeight="1">
+    <row r="135" ht="165" customHeight="1">
       <c r="A135" s="84" t="inlineStr">
         <is>
-          <t>Área neta por rejilla de salida</t>
+          <t>Diámetro del impulsor seleccionado</t>
         </is>
       </c>
       <c r="B135" s="85" t="n"/>
       <c r="C135" s="85" t="n"/>
       <c r="D135" s="85" t="n"/>
-      <c r="E135" s="92">
-        <f>J58</f>
-        <v/>
+      <c r="E135" s="92" t="n">
+        <v>0.5600000000000001</v>
       </c>
       <c r="F135" s="93" t="n"/>
       <c r="G135" s="93" t="n"/>
       <c r="H135" s="93" t="n"/>
       <c r="I135" s="86" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
       <c r="J135" s="85" t="n"/>
@@ -7181,7 +7185,7 @@
       <c r="L135" s="85" t="n"/>
       <c r="M135" s="84" t="inlineStr">
         <is>
-          <t>Cada rejilla</t>
+          <t>Ø560 mm — uniformidad con montaje típico de planta (REV2)</t>
         </is>
       </c>
       <c r="N135" s="85" t="n"/>
@@ -7190,14 +7194,14 @@
     <row r="136" ht="75" customHeight="1">
       <c r="A136" s="84" t="inlineStr">
         <is>
-          <t>Altura de rejilla de salida</t>
+          <t>Área de boca real (Ø560 mm)</t>
         </is>
       </c>
       <c r="B136" s="85" t="n"/>
       <c r="C136" s="85" t="n"/>
       <c r="D136" s="85" t="n"/>
       <c r="E136" s="92">
-        <f>J61</f>
+        <f>PI()*(0.56/2)^2</f>
         <v/>
       </c>
       <c r="F136" s="93" t="n"/>
@@ -7205,7 +7209,7 @@
       <c r="H136" s="93" t="n"/>
       <c r="I136" s="86" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="J136" s="85" t="n"/>
@@ -7213,23 +7217,23 @@
       <c r="L136" s="85" t="n"/>
       <c r="M136" s="84" t="inlineStr">
         <is>
-          <t>Dimensiones para CFD</t>
+          <t>π × (D/2)²</t>
         </is>
       </c>
       <c r="N136" s="85" t="n"/>
       <c r="O136" s="85" t="n"/>
     </row>
-    <row r="137" ht="75" customHeight="1">
+    <row r="137" ht="90" customHeight="1">
       <c r="A137" s="84" t="inlineStr">
         <is>
-          <t>Ancho de rejilla de salida</t>
+          <t>Velocidad real en boca (Ø560 mm)</t>
         </is>
       </c>
       <c r="B137" s="85" t="n"/>
       <c r="C137" s="85" t="n"/>
       <c r="D137" s="85" t="n"/>
       <c r="E137" s="92">
-        <f>J62</f>
+        <f>J50/(PI()*(0.56/2)^2)</f>
         <v/>
       </c>
       <c r="F137" s="93" t="n"/>
@@ -7237,7 +7241,7 @@
       <c r="H137" s="93" t="n"/>
       <c r="I137" s="86" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>m/s</t>
         </is>
       </c>
       <c r="J137" s="85" t="n"/>
@@ -7245,7 +7249,7 @@
       <c r="L137" s="85" t="n"/>
       <c r="M137" s="84" t="inlineStr">
         <is>
-          <t>Dimensiones para CFD</t>
+          <t>Q_s / A_boca real ≈ 4,33 m/s</t>
         </is>
       </c>
       <c r="N137" s="85" t="n"/>
@@ -7254,14 +7258,14 @@
     <row r="138" ht="75" customHeight="1">
       <c r="A138" s="84" t="inlineStr">
         <is>
-          <t>Velocidad de exfiltración</t>
+          <t>Velocidad de impulsión</t>
         </is>
       </c>
       <c r="B138" s="85" t="n"/>
       <c r="C138" s="85" t="n"/>
       <c r="D138" s="85" t="n"/>
       <c r="E138" s="92">
-        <f>G33</f>
+        <f>G32</f>
         <v/>
       </c>
       <c r="F138" s="93" t="n"/>
@@ -7277,7 +7281,7 @@
       <c r="L138" s="85" t="n"/>
       <c r="M138" s="84" t="inlineStr">
         <is>
-          <t>Condición de salida CFD</t>
+          <t>Condición de entrada CFD</t>
         </is>
       </c>
       <c r="N138" s="85" t="n"/>
@@ -7286,14 +7290,14 @@
     <row r="139" ht="105" customHeight="1">
       <c r="A139" s="84" t="inlineStr">
         <is>
-          <t>Pérdida de presión en rejillas</t>
+          <t>Área neta total de rejillas de salida</t>
         </is>
       </c>
       <c r="B139" s="85" t="n"/>
       <c r="C139" s="85" t="n"/>
       <c r="D139" s="85" t="n"/>
       <c r="E139" s="92">
-        <f>J63</f>
+        <f>J57</f>
         <v/>
       </c>
       <c r="F139" s="93" t="n"/>
@@ -7301,7 +7305,7 @@
       <c r="H139" s="93" t="n"/>
       <c r="I139" s="86" t="inlineStr">
         <is>
-          <t>Pa</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="J139" s="85" t="n"/>
@@ -7309,34 +7313,227 @@
       <c r="L139" s="85" t="n"/>
       <c r="M139" s="84" t="inlineStr">
         <is>
-          <t>Descarga libre a atmósfera, Cd=0.6</t>
+          <t>A v=3 m/s</t>
         </is>
       </c>
       <c r="N139" s="85" t="n"/>
       <c r="O139" s="85" t="n"/>
     </row>
-    <row r="140" ht="15" customHeight="1"/>
-    <row r="141" ht="15" customHeight="1">
-      <c r="A141" s="82" t="inlineStr">
+    <row r="140" ht="75" customHeight="1">
+      <c r="A140" s="84" t="inlineStr">
+        <is>
+          <t>Número de rejillas de salida</t>
+        </is>
+      </c>
+      <c r="B140" s="85" t="n"/>
+      <c r="C140" s="85" t="n"/>
+      <c r="D140" s="85" t="n"/>
+      <c r="E140" s="92">
+        <f>G34</f>
+        <v/>
+      </c>
+      <c r="F140" s="93" t="n"/>
+      <c r="G140" s="93" t="n"/>
+      <c r="H140" s="93" t="n"/>
+      <c r="I140" s="86" t="inlineStr">
+        <is>
+          <t>unid.</t>
+        </is>
+      </c>
+      <c r="J140" s="85" t="n"/>
+      <c r="K140" s="85" t="n"/>
+      <c r="L140" s="85" t="n"/>
+      <c r="M140" s="84" t="inlineStr">
+        <is>
+          <t>Distribución propuesta</t>
+        </is>
+      </c>
+      <c r="N140" s="85" t="n"/>
+      <c r="O140" s="85" t="n"/>
+    </row>
+    <row r="141" ht="90" customHeight="1">
+      <c r="A141" s="84" t="inlineStr">
+        <is>
+          <t>Área neta por rejilla de salida</t>
+        </is>
+      </c>
+      <c r="B141" s="85" t="n"/>
+      <c r="C141" s="85" t="n"/>
+      <c r="D141" s="85" t="n"/>
+      <c r="E141" s="92">
+        <f>J58</f>
+        <v/>
+      </c>
+      <c r="F141" s="93" t="n"/>
+      <c r="G141" s="93" t="n"/>
+      <c r="H141" s="93" t="n"/>
+      <c r="I141" s="86" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="J141" s="85" t="n"/>
+      <c r="K141" s="85" t="n"/>
+      <c r="L141" s="85" t="n"/>
+      <c r="M141" s="84" t="inlineStr">
+        <is>
+          <t>Cada rejilla</t>
+        </is>
+      </c>
+      <c r="N141" s="85" t="n"/>
+      <c r="O141" s="85" t="n"/>
+    </row>
+    <row r="142" ht="75" customHeight="1">
+      <c r="A142" s="84" t="inlineStr">
+        <is>
+          <t>Altura de rejilla de salida</t>
+        </is>
+      </c>
+      <c r="B142" s="85" t="n"/>
+      <c r="C142" s="85" t="n"/>
+      <c r="D142" s="85" t="n"/>
+      <c r="E142" s="92">
+        <f>J61</f>
+        <v/>
+      </c>
+      <c r="F142" s="93" t="n"/>
+      <c r="G142" s="93" t="n"/>
+      <c r="H142" s="93" t="n"/>
+      <c r="I142" s="86" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="J142" s="85" t="n"/>
+      <c r="K142" s="85" t="n"/>
+      <c r="L142" s="85" t="n"/>
+      <c r="M142" s="84" t="inlineStr">
+        <is>
+          <t>Dimensiones para CFD</t>
+        </is>
+      </c>
+      <c r="N142" s="85" t="n"/>
+      <c r="O142" s="85" t="n"/>
+    </row>
+    <row r="143" ht="75" customHeight="1">
+      <c r="A143" s="84" t="inlineStr">
+        <is>
+          <t>Ancho de rejilla de salida</t>
+        </is>
+      </c>
+      <c r="B143" s="85" t="n"/>
+      <c r="C143" s="85" t="n"/>
+      <c r="D143" s="85" t="n"/>
+      <c r="E143" s="92">
+        <f>J62</f>
+        <v/>
+      </c>
+      <c r="F143" s="93" t="n"/>
+      <c r="G143" s="93" t="n"/>
+      <c r="H143" s="93" t="n"/>
+      <c r="I143" s="86" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="J143" s="85" t="n"/>
+      <c r="K143" s="85" t="n"/>
+      <c r="L143" s="85" t="n"/>
+      <c r="M143" s="84" t="inlineStr">
+        <is>
+          <t>Dimensiones para CFD</t>
+        </is>
+      </c>
+      <c r="N143" s="85" t="n"/>
+      <c r="O143" s="85" t="n"/>
+    </row>
+    <row r="144" ht="75" customHeight="1">
+      <c r="A144" s="84" t="inlineStr">
+        <is>
+          <t>Velocidad de exfiltración</t>
+        </is>
+      </c>
+      <c r="B144" s="85" t="n"/>
+      <c r="C144" s="85" t="n"/>
+      <c r="D144" s="85" t="n"/>
+      <c r="E144" s="92">
+        <f>G33</f>
+        <v/>
+      </c>
+      <c r="F144" s="93" t="n"/>
+      <c r="G144" s="93" t="n"/>
+      <c r="H144" s="93" t="n"/>
+      <c r="I144" s="86" t="inlineStr">
+        <is>
+          <t>m/s</t>
+        </is>
+      </c>
+      <c r="J144" s="85" t="n"/>
+      <c r="K144" s="85" t="n"/>
+      <c r="L144" s="85" t="n"/>
+      <c r="M144" s="84" t="inlineStr">
+        <is>
+          <t>Condición de salida CFD</t>
+        </is>
+      </c>
+      <c r="N144" s="85" t="n"/>
+      <c r="O144" s="85" t="n"/>
+    </row>
+    <row r="145" ht="105" customHeight="1">
+      <c r="A145" s="84" t="inlineStr">
+        <is>
+          <t>Pérdida de presión en rejillas</t>
+        </is>
+      </c>
+      <c r="B145" s="85" t="n"/>
+      <c r="C145" s="85" t="n"/>
+      <c r="D145" s="85" t="n"/>
+      <c r="E145" s="92">
+        <f>J63</f>
+        <v/>
+      </c>
+      <c r="F145" s="93" t="n"/>
+      <c r="G145" s="93" t="n"/>
+      <c r="H145" s="93" t="n"/>
+      <c r="I145" s="86" t="inlineStr">
+        <is>
+          <t>Pa</t>
+        </is>
+      </c>
+      <c r="J145" s="85" t="n"/>
+      <c r="K145" s="85" t="n"/>
+      <c r="L145" s="85" t="n"/>
+      <c r="M145" s="84" t="inlineStr">
+        <is>
+          <t>Descarga libre a atmósfera, Cd=0.6</t>
+        </is>
+      </c>
+      <c r="N145" s="85" t="n"/>
+      <c r="O145" s="85" t="n"/>
+    </row>
+    <row r="146" ht="15" customHeight="1"/>
+    <row r="147" ht="15" customHeight="1">
+      <c r="A147" s="82" t="inlineStr">
         <is>
           <t>Nota:</t>
         </is>
       </c>
     </row>
-    <row r="142" ht="210" customHeight="1">
-      <c r="A142" s="87" t="inlineStr">
+    <row r="148" ht="210" customHeight="1">
+      <c r="A148" s="87" t="inlineStr">
         <is>
           <t>Sección con fórmulas vivas que referencian las secciones 3. DESARROLLO DE CÁLCULOS y 2. PARÁMETROS DE ENTRADA de esta misma hoja. Si modifica las entradas, esta vista y la sección 4. RESULTADOS se actualizan automáticamente.</t>
         </is>
       </c>
     </row>
-    <row r="143" ht="15" customHeight="1"/>
-    <row r="144" ht="15" customHeight="1"/>
+    <row r="149" ht="15" customHeight="1"/>
+    <row r="150" ht="15" customHeight="1"/>
   </sheetData>
-  <mergeCells count="445">
+  <mergeCells count="469">
     <mergeCell ref="A25:O25"/>
     <mergeCell ref="G112:I112"/>
     <mergeCell ref="N113:O113"/>
+    <mergeCell ref="D116:F116"/>
     <mergeCell ref="G62:I62"/>
     <mergeCell ref="A134:D134"/>
     <mergeCell ref="J59:K59"/>
@@ -7345,23 +7542,19 @@
     <mergeCell ref="D47:F47"/>
     <mergeCell ref="A57:C57"/>
     <mergeCell ref="A113:C113"/>
+    <mergeCell ref="M145:O145"/>
     <mergeCell ref="A73:D73"/>
     <mergeCell ref="M76:O76"/>
     <mergeCell ref="A52:C52"/>
-    <mergeCell ref="E88:H88"/>
-    <mergeCell ref="A124:D124"/>
     <mergeCell ref="E82:H82"/>
     <mergeCell ref="A34:C34"/>
     <mergeCell ref="A40:O40"/>
     <mergeCell ref="E128:H128"/>
     <mergeCell ref="G36:I36"/>
     <mergeCell ref="A49:C49"/>
-    <mergeCell ref="A107:O107"/>
-    <mergeCell ref="A110:C110"/>
     <mergeCell ref="J62:K62"/>
     <mergeCell ref="A17:D17"/>
     <mergeCell ref="M94:O94"/>
-    <mergeCell ref="I123:L123"/>
     <mergeCell ref="A126:D126"/>
     <mergeCell ref="M31:O31"/>
     <mergeCell ref="J57:K57"/>
@@ -7369,9 +7562,9 @@
     <mergeCell ref="A55:C55"/>
     <mergeCell ref="E75:H75"/>
     <mergeCell ref="M95:O95"/>
-    <mergeCell ref="M89:O89"/>
     <mergeCell ref="E12:H12"/>
-    <mergeCell ref="A141:O141"/>
+    <mergeCell ref="N115:O115"/>
+    <mergeCell ref="A142:D142"/>
     <mergeCell ref="A29:C29"/>
     <mergeCell ref="M97:O97"/>
     <mergeCell ref="G51:I51"/>
@@ -7383,24 +7576,24 @@
     <mergeCell ref="I70:L70"/>
     <mergeCell ref="A31:C31"/>
     <mergeCell ref="A58:C58"/>
-    <mergeCell ref="A102:O104"/>
+    <mergeCell ref="N116:O116"/>
     <mergeCell ref="I134:L134"/>
     <mergeCell ref="A137:D137"/>
     <mergeCell ref="A60:C60"/>
     <mergeCell ref="I96:L96"/>
     <mergeCell ref="I71:L71"/>
     <mergeCell ref="A74:D74"/>
+    <mergeCell ref="A145:D145"/>
     <mergeCell ref="A139:D139"/>
-    <mergeCell ref="E90:H90"/>
     <mergeCell ref="I98:L98"/>
     <mergeCell ref="A76:D76"/>
     <mergeCell ref="A41:O41"/>
+    <mergeCell ref="A140:D140"/>
     <mergeCell ref="A50:C50"/>
     <mergeCell ref="L47:M47"/>
     <mergeCell ref="G58:I58"/>
+    <mergeCell ref="M85:O85"/>
     <mergeCell ref="A92:D92"/>
-    <mergeCell ref="G110:I110"/>
-    <mergeCell ref="I124:L124"/>
     <mergeCell ref="D51:F51"/>
     <mergeCell ref="A94:D94"/>
     <mergeCell ref="M32:O32"/>
@@ -7408,6 +7601,7 @@
     <mergeCell ref="A69:D69"/>
     <mergeCell ref="I126:L126"/>
     <mergeCell ref="L50:M50"/>
+    <mergeCell ref="A87:D87"/>
     <mergeCell ref="M96:O96"/>
     <mergeCell ref="A9:O9"/>
     <mergeCell ref="A133:D133"/>
@@ -7417,13 +7611,14 @@
     <mergeCell ref="E84:H84"/>
     <mergeCell ref="E78:H78"/>
     <mergeCell ref="L52:M52"/>
-    <mergeCell ref="A89:D89"/>
     <mergeCell ref="M98:O98"/>
     <mergeCell ref="A11:O11"/>
     <mergeCell ref="E15:H15"/>
+    <mergeCell ref="E86:H86"/>
     <mergeCell ref="E80:H80"/>
+    <mergeCell ref="I142:L142"/>
     <mergeCell ref="A65:O65"/>
-    <mergeCell ref="N109:O109"/>
+    <mergeCell ref="E144:H144"/>
     <mergeCell ref="I79:L79"/>
     <mergeCell ref="N47:O47"/>
     <mergeCell ref="I73:L73"/>
@@ -7444,8 +7639,8 @@
     <mergeCell ref="M93:O93"/>
     <mergeCell ref="I92:L92"/>
     <mergeCell ref="A95:D95"/>
+    <mergeCell ref="N114:O114"/>
     <mergeCell ref="I67:L67"/>
-    <mergeCell ref="A122:D122"/>
     <mergeCell ref="A97:D97"/>
     <mergeCell ref="A46:C46"/>
     <mergeCell ref="A72:D72"/>
@@ -7455,13 +7650,14 @@
     <mergeCell ref="E125:H125"/>
     <mergeCell ref="N3:O3"/>
     <mergeCell ref="D37:F37"/>
+    <mergeCell ref="A104:O104"/>
     <mergeCell ref="N46:O46"/>
     <mergeCell ref="I81:L81"/>
     <mergeCell ref="E129:H129"/>
     <mergeCell ref="N61:O61"/>
     <mergeCell ref="N5:O5"/>
-    <mergeCell ref="A106:O106"/>
     <mergeCell ref="N48:O48"/>
+    <mergeCell ref="I145:L145"/>
     <mergeCell ref="E131:H131"/>
     <mergeCell ref="I16:L16"/>
     <mergeCell ref="I76:L76"/>
@@ -7473,48 +7669,45 @@
     <mergeCell ref="M67:O67"/>
     <mergeCell ref="E99:H99"/>
     <mergeCell ref="M132:O132"/>
-    <mergeCell ref="J110:K110"/>
-    <mergeCell ref="L110:M110"/>
+    <mergeCell ref="A85:D85"/>
     <mergeCell ref="M69:O69"/>
+    <mergeCell ref="E101:H101"/>
     <mergeCell ref="D27:F27"/>
     <mergeCell ref="G28:I28"/>
+    <mergeCell ref="E100:H100"/>
     <mergeCell ref="N51:O51"/>
     <mergeCell ref="E136:H136"/>
     <mergeCell ref="G30:I30"/>
     <mergeCell ref="I94:L94"/>
-    <mergeCell ref="A101:O101"/>
     <mergeCell ref="M37:O37"/>
+    <mergeCell ref="E102:H102"/>
     <mergeCell ref="A32:C32"/>
     <mergeCell ref="J49:K49"/>
     <mergeCell ref="I77:L77"/>
     <mergeCell ref="I133:L133"/>
     <mergeCell ref="I95:L95"/>
     <mergeCell ref="A98:D98"/>
-    <mergeCell ref="I89:L89"/>
     <mergeCell ref="M14:O14"/>
     <mergeCell ref="E127:H127"/>
     <mergeCell ref="G54:I54"/>
     <mergeCell ref="A20:O20"/>
     <mergeCell ref="I135:L135"/>
-    <mergeCell ref="M122:O122"/>
     <mergeCell ref="G56:I56"/>
     <mergeCell ref="I72:L72"/>
-    <mergeCell ref="D109:F109"/>
     <mergeCell ref="N6:O6"/>
     <mergeCell ref="J37:L37"/>
     <mergeCell ref="D46:F46"/>
-    <mergeCell ref="D111:F111"/>
     <mergeCell ref="N4:O4"/>
     <mergeCell ref="M138:O138"/>
     <mergeCell ref="I17:L17"/>
-    <mergeCell ref="I88:L88"/>
     <mergeCell ref="A91:D91"/>
-    <mergeCell ref="E124:H124"/>
     <mergeCell ref="I82:L82"/>
+    <mergeCell ref="M140:O140"/>
     <mergeCell ref="G34:I34"/>
     <mergeCell ref="A93:D93"/>
     <mergeCell ref="A68:D68"/>
     <mergeCell ref="M77:O77"/>
+    <mergeCell ref="A105:O107"/>
     <mergeCell ref="M133:O133"/>
     <mergeCell ref="J32:L32"/>
     <mergeCell ref="M33:O33"/>
@@ -7523,11 +7716,10 @@
     <mergeCell ref="M135:O135"/>
     <mergeCell ref="G29:I29"/>
     <mergeCell ref="D33:F33"/>
-    <mergeCell ref="E123:H123"/>
-    <mergeCell ref="A115:O115"/>
     <mergeCell ref="G31:I31"/>
     <mergeCell ref="D35:F35"/>
     <mergeCell ref="D59:F59"/>
+    <mergeCell ref="M87:O87"/>
     <mergeCell ref="J113:K113"/>
     <mergeCell ref="L113:M113"/>
     <mergeCell ref="D34:F34"/>
@@ -7535,53 +7727,61 @@
     <mergeCell ref="I97:L97"/>
     <mergeCell ref="J50:K50"/>
     <mergeCell ref="A12:D12"/>
+    <mergeCell ref="J115:K115"/>
+    <mergeCell ref="L115:M115"/>
     <mergeCell ref="D36:F36"/>
-    <mergeCell ref="M88:O88"/>
     <mergeCell ref="J52:K52"/>
     <mergeCell ref="M82:O82"/>
     <mergeCell ref="A14:D14"/>
     <mergeCell ref="E70:H70"/>
     <mergeCell ref="G57:I57"/>
     <mergeCell ref="D61:F61"/>
-    <mergeCell ref="M90:O90"/>
+    <mergeCell ref="J116:K116"/>
     <mergeCell ref="D48:F48"/>
     <mergeCell ref="G49:I49"/>
     <mergeCell ref="E134:H134"/>
     <mergeCell ref="D112:F112"/>
+    <mergeCell ref="A116:C116"/>
     <mergeCell ref="D62:F62"/>
     <mergeCell ref="A130:D130"/>
     <mergeCell ref="D56:F56"/>
     <mergeCell ref="A53:C53"/>
-    <mergeCell ref="A109:C109"/>
+    <mergeCell ref="D114:F114"/>
     <mergeCell ref="N1:O1"/>
     <mergeCell ref="A138:D138"/>
     <mergeCell ref="A132:D132"/>
     <mergeCell ref="E83:H83"/>
-    <mergeCell ref="A111:C111"/>
+    <mergeCell ref="M141:O141"/>
+    <mergeCell ref="E140:H140"/>
     <mergeCell ref="J63:K63"/>
     <mergeCell ref="I91:L91"/>
     <mergeCell ref="L63:M63"/>
+    <mergeCell ref="I85:L85"/>
     <mergeCell ref="M34:O34"/>
     <mergeCell ref="A48:C48"/>
     <mergeCell ref="J47:K47"/>
     <mergeCell ref="M83:O83"/>
-    <mergeCell ref="J109:K109"/>
+    <mergeCell ref="M143:O143"/>
     <mergeCell ref="I93:L93"/>
+    <mergeCell ref="A110:O110"/>
+    <mergeCell ref="A148:O150"/>
+    <mergeCell ref="G116:I116"/>
     <mergeCell ref="M78:O78"/>
     <mergeCell ref="D49:F49"/>
     <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A118:O118"/>
     <mergeCell ref="J35:L35"/>
     <mergeCell ref="A13:D13"/>
     <mergeCell ref="J60:K60"/>
+    <mergeCell ref="L116:M116"/>
     <mergeCell ref="J53:K53"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="E71:H71"/>
+    <mergeCell ref="E142:H142"/>
     <mergeCell ref="G63:I63"/>
     <mergeCell ref="G50:I50"/>
     <mergeCell ref="A63:C63"/>
-    <mergeCell ref="N111:O111"/>
     <mergeCell ref="E79:H79"/>
-    <mergeCell ref="L109:M109"/>
     <mergeCell ref="E73:H73"/>
     <mergeCell ref="M131:O131"/>
     <mergeCell ref="A44:O44"/>
@@ -7593,32 +7793,27 @@
     <mergeCell ref="J58:K58"/>
     <mergeCell ref="B1:B5"/>
     <mergeCell ref="D57:F57"/>
+    <mergeCell ref="A141:D141"/>
     <mergeCell ref="I132:L132"/>
     <mergeCell ref="A135:D135"/>
     <mergeCell ref="M84:O84"/>
     <mergeCell ref="M75:O75"/>
     <mergeCell ref="M15:O15"/>
+    <mergeCell ref="M86:O86"/>
     <mergeCell ref="M80:O80"/>
-    <mergeCell ref="A86:O86"/>
     <mergeCell ref="A42:O42"/>
     <mergeCell ref="G55:I55"/>
-    <mergeCell ref="A116:O118"/>
     <mergeCell ref="E67:H67"/>
-    <mergeCell ref="A88:D88"/>
-    <mergeCell ref="D110:F110"/>
     <mergeCell ref="D60:F60"/>
+    <mergeCell ref="E87:H87"/>
     <mergeCell ref="I125:L125"/>
     <mergeCell ref="A128:D128"/>
-    <mergeCell ref="A90:D90"/>
     <mergeCell ref="A51:C51"/>
     <mergeCell ref="L59:M59"/>
-    <mergeCell ref="I122:L122"/>
     <mergeCell ref="A136:D136"/>
     <mergeCell ref="J46:K46"/>
     <mergeCell ref="I127:L127"/>
     <mergeCell ref="L46:M46"/>
-    <mergeCell ref="L111:M111"/>
-    <mergeCell ref="A142:O144"/>
     <mergeCell ref="M70:O70"/>
     <mergeCell ref="A129:D129"/>
     <mergeCell ref="M35:O35"/>
@@ -7640,11 +7835,14 @@
     <mergeCell ref="E18:H18"/>
     <mergeCell ref="I69:L69"/>
     <mergeCell ref="A83:D83"/>
+    <mergeCell ref="I140:L140"/>
+    <mergeCell ref="A143:D143"/>
     <mergeCell ref="D58:F58"/>
     <mergeCell ref="A62:C62"/>
     <mergeCell ref="A28:C28"/>
     <mergeCell ref="E92:H92"/>
     <mergeCell ref="M125:O125"/>
+    <mergeCell ref="L114:M114"/>
     <mergeCell ref="A78:D78"/>
     <mergeCell ref="A30:C30"/>
     <mergeCell ref="N59:O59"/>
@@ -7654,38 +7852,46 @@
     <mergeCell ref="A1:A5"/>
     <mergeCell ref="A80:D80"/>
     <mergeCell ref="A61:C61"/>
+    <mergeCell ref="I87:L87"/>
     <mergeCell ref="E95:H95"/>
-    <mergeCell ref="E89:H89"/>
+    <mergeCell ref="A119:O121"/>
     <mergeCell ref="A54:C54"/>
     <mergeCell ref="M13:O13"/>
     <mergeCell ref="A27:C27"/>
     <mergeCell ref="A56:C56"/>
-    <mergeCell ref="N110:O110"/>
     <mergeCell ref="E72:H72"/>
+    <mergeCell ref="A89:O89"/>
     <mergeCell ref="I128:L128"/>
     <mergeCell ref="M36:O36"/>
     <mergeCell ref="L62:M62"/>
+    <mergeCell ref="M101:O101"/>
     <mergeCell ref="N62:O62"/>
+    <mergeCell ref="M100:O100"/>
+    <mergeCell ref="A147:O147"/>
     <mergeCell ref="E17:H17"/>
     <mergeCell ref="E126:H126"/>
     <mergeCell ref="L51:M51"/>
+    <mergeCell ref="M102:O102"/>
     <mergeCell ref="N57:O57"/>
     <mergeCell ref="A84:D84"/>
+    <mergeCell ref="I141:L141"/>
     <mergeCell ref="I75:L75"/>
     <mergeCell ref="A75:D75"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="I12:L12"/>
+    <mergeCell ref="A86:D86"/>
+    <mergeCell ref="I143:L143"/>
     <mergeCell ref="I14:L14"/>
+    <mergeCell ref="A144:D144"/>
     <mergeCell ref="M128:O128"/>
     <mergeCell ref="J27:L27"/>
     <mergeCell ref="I78:L78"/>
     <mergeCell ref="A81:D81"/>
-    <mergeCell ref="A120:O120"/>
     <mergeCell ref="E97:H97"/>
     <mergeCell ref="D28:F28"/>
     <mergeCell ref="E96:H96"/>
+    <mergeCell ref="E145:H145"/>
     <mergeCell ref="E139:H139"/>
-    <mergeCell ref="I90:L90"/>
     <mergeCell ref="D30:F30"/>
     <mergeCell ref="C2:L3"/>
     <mergeCell ref="I136:L136"/>
@@ -7694,13 +7900,16 @@
     <mergeCell ref="D29:F29"/>
     <mergeCell ref="I129:L129"/>
     <mergeCell ref="A99:D99"/>
+    <mergeCell ref="G115:I115"/>
     <mergeCell ref="I131:L131"/>
-    <mergeCell ref="M123:O123"/>
+    <mergeCell ref="A101:D101"/>
+    <mergeCell ref="A123:O123"/>
     <mergeCell ref="I83:L83"/>
     <mergeCell ref="G37:I37"/>
     <mergeCell ref="N63:O63"/>
     <mergeCell ref="E91:H91"/>
     <mergeCell ref="N50:O50"/>
+    <mergeCell ref="E85:H85"/>
     <mergeCell ref="A125:D125"/>
     <mergeCell ref="M28:O28"/>
     <mergeCell ref="I13:L13"/>
@@ -7710,14 +7919,16 @@
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="M136:O136"/>
     <mergeCell ref="I15:L15"/>
-    <mergeCell ref="E122:H122"/>
+    <mergeCell ref="I86:L86"/>
     <mergeCell ref="I80:L80"/>
     <mergeCell ref="M29:O29"/>
     <mergeCell ref="M134:O134"/>
     <mergeCell ref="G32:I32"/>
     <mergeCell ref="J33:L33"/>
+    <mergeCell ref="I144:L144"/>
     <mergeCell ref="D54:F54"/>
     <mergeCell ref="M71:O71"/>
+    <mergeCell ref="J114:K114"/>
     <mergeCell ref="G27:I27"/>
     <mergeCell ref="J28:L28"/>
     <mergeCell ref="D31:F31"/>
@@ -7725,10 +7936,10 @@
     <mergeCell ref="A71:D71"/>
     <mergeCell ref="J30:L30"/>
     <mergeCell ref="N55:O55"/>
-    <mergeCell ref="J111:K111"/>
     <mergeCell ref="D32:F32"/>
+    <mergeCell ref="A100:D100"/>
     <mergeCell ref="I99:L99"/>
-    <mergeCell ref="M124:O124"/>
+    <mergeCell ref="A102:D102"/>
     <mergeCell ref="I74:L74"/>
     <mergeCell ref="A77:D77"/>
     <mergeCell ref="M17:O17"/>
@@ -7736,20 +7947,25 @@
     <mergeCell ref="E68:H68"/>
     <mergeCell ref="M126:O126"/>
     <mergeCell ref="E130:H130"/>
-    <mergeCell ref="G109:I109"/>
+    <mergeCell ref="A109:O109"/>
     <mergeCell ref="G47:I47"/>
     <mergeCell ref="A112:C112"/>
     <mergeCell ref="D113:F113"/>
     <mergeCell ref="E135:H135"/>
+    <mergeCell ref="E141:H141"/>
     <mergeCell ref="E132:H132"/>
     <mergeCell ref="G46:I46"/>
     <mergeCell ref="D50:F50"/>
-    <mergeCell ref="G111:I111"/>
+    <mergeCell ref="E143:H143"/>
+    <mergeCell ref="A114:C114"/>
+    <mergeCell ref="D115:F115"/>
     <mergeCell ref="C1:L1"/>
+    <mergeCell ref="M142:O142"/>
     <mergeCell ref="M129:O129"/>
     <mergeCell ref="M79:O79"/>
     <mergeCell ref="J34:L34"/>
     <mergeCell ref="M73:O73"/>
+    <mergeCell ref="M144:O144"/>
     <mergeCell ref="M137:O137"/>
     <mergeCell ref="J36:L36"/>
     <mergeCell ref="A96:D96"/>
@@ -7757,12 +7973,15 @@
     <mergeCell ref="M139:O139"/>
     <mergeCell ref="G33:I33"/>
     <mergeCell ref="A33:C33"/>
+    <mergeCell ref="G114:I114"/>
     <mergeCell ref="J31:L31"/>
     <mergeCell ref="G35:I35"/>
     <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A123:D123"/>
+    <mergeCell ref="A115:C115"/>
+    <mergeCell ref="I101:L101"/>
     <mergeCell ref="J54:K54"/>
     <mergeCell ref="L54:M54"/>
+    <mergeCell ref="I100:L100"/>
     <mergeCell ref="E138:H138"/>
     <mergeCell ref="G59:I59"/>
     <mergeCell ref="D63:F63"/>
@@ -7771,6 +7990,7 @@
     <mergeCell ref="L56:M56"/>
     <mergeCell ref="A18:D18"/>
     <mergeCell ref="E69:H69"/>
+    <mergeCell ref="I102:L102"/>
     <mergeCell ref="C4:L6"/>
     <mergeCell ref="G61:I61"/>
     <mergeCell ref="L49:M49"/>

</xml_diff>

<commit_message>
REV0 unica + geometria Excel 35/50: entregables en Revision CERO (0), columnas 35 y filas 50
- Geometria Excel fija (instruccion cliente): ANCHO_COLUMNAS=[35]*15, ALTURA_LINEA/ALTURA_MINIMA=50 en scripts/estilos_excel.py; portadas y encabezado corporativo conservan plantilla
- REV0 unica (GP-N-09): eliminadas referencias REV1/REV2 de hojas de datos, listado, informe investigacion, INF-001/002 (tablas de revision solo REV0, macros descRevUno.. eliminadas), pdf_dts001, emitir, codificacion, dashboard, bases_diseno.yaml
- Re-emitidos 7 entregables + PDF DTS-001; verificacion: 0 coincidencias REV1/REV2 en Emisiones/
- Retirado P2437-HV-CAL-001.pdf (exportacion manual obsoleta)
- Memoria: contexto.md, vault (estado, bases, bitacora 2026-07-28, decision rev0-unica)
</commit_message>
<xml_diff>
--- a/Emisiones/2.0 HV-MEMORIAS DE CALCULO/P2437-HV-CAL-001.xlsx
+++ b/Emisiones/2.0 HV-MEMORIAS DE CALCULO/P2437-HV-CAL-001.xlsx
@@ -3751,21 +3751,21 @@
   <dimension ref="A1:O150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="49" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="35" customWidth="1" min="11" max="11"/>
+    <col width="35" customWidth="1" min="12" max="12"/>
+    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="35" customWidth="1" min="14" max="14"/>
+    <col width="35" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
@@ -4093,22 +4093,22 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" ht="228" customHeight="1">
+    <row r="9" ht="100" customHeight="1">
       <c r="A9" s="81" t="inlineStr">
         <is>
           <t>1. DATOS GENERALES — MEMORIA DE CÁLCULO, SISTEMA DE VENTILACIÓN</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="38" customHeight="1"/>
-    <row r="11" ht="76" customHeight="1">
+    <row r="10" ht="50" customHeight="1"/>
+    <row r="11" ht="50" customHeight="1">
       <c r="A11" s="81" t="inlineStr">
         <is>
           <t>Información del proyecto</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="38" customHeight="1">
+    <row r="12" ht="50" customHeight="1">
       <c r="A12" s="82" t="inlineStr">
         <is>
           <t>Concepto</t>
@@ -4141,7 +4141,7 @@
       <c r="N12" s="82" t="n"/>
       <c r="O12" s="82" t="n"/>
     </row>
-    <row r="13" ht="152" customHeight="1">
+    <row r="13" ht="100" customHeight="1">
       <c r="A13" s="83" t="inlineStr">
         <is>
           <t>Nombre del proyecto</t>
@@ -4174,7 +4174,7 @@
       <c r="N13" s="84" t="n"/>
       <c r="O13" s="84" t="n"/>
     </row>
-    <row r="14" ht="114" customHeight="1">
+    <row r="14" ht="100" customHeight="1">
       <c r="A14" s="83" t="inlineStr">
         <is>
           <t>Ubicación</t>
@@ -4207,7 +4207,7 @@
       <c r="N14" s="84" t="n"/>
       <c r="O14" s="84" t="n"/>
     </row>
-    <row r="15" ht="114" customHeight="1">
+    <row r="15" ht="50" customHeight="1">
       <c r="A15" s="83" t="inlineStr">
         <is>
           <t>Volumen efectivo del laboratorio (V)</t>
@@ -4240,7 +4240,7 @@
       <c r="N15" s="84" t="n"/>
       <c r="O15" s="84" t="n"/>
     </row>
-    <row r="16" ht="76" customHeight="1">
+    <row r="16" ht="100" customHeight="1">
       <c r="A16" s="83" t="inlineStr">
         <is>
           <t>Renovaciones de aire (N)</t>
@@ -4273,7 +4273,7 @@
       <c r="N16" s="84" t="n"/>
       <c r="O16" s="84" t="n"/>
     </row>
-    <row r="17" ht="152" customHeight="1">
+    <row r="17" ht="150" customHeight="1">
       <c r="A17" s="83" t="inlineStr">
         <is>
           <t>Objetivo</t>
@@ -4300,13 +4300,13 @@
       <c r="L17" s="84" t="n"/>
       <c r="M17" s="83" t="inlineStr">
         <is>
-          <t>12 ACH, MERV 13-14; sin presurización (REV1)</t>
+          <t>12 ACH, MERV 13-14; sin presurización</t>
         </is>
       </c>
       <c r="N17" s="84" t="n"/>
       <c r="O17" s="84" t="n"/>
     </row>
-    <row r="18" ht="266" customHeight="1">
+    <row r="18" ht="350" customHeight="1">
       <c r="A18" s="83" t="inlineStr">
         <is>
           <t>Estrategia</t>
@@ -4333,39 +4333,39 @@
       <c r="L18" s="84" t="n"/>
       <c r="M18" s="83" t="inlineStr">
         <is>
-          <t>Sin ductos de impulsión; montaje uniforme con la planta (REV2)</t>
+          <t>Sin ductos de impulsión; montaje uniforme con la planta</t>
         </is>
       </c>
       <c r="N18" s="84" t="n"/>
       <c r="O18" s="84" t="n"/>
     </row>
-    <row r="19" ht="38" customHeight="1"/>
-    <row r="20" ht="76" customHeight="1">
+    <row r="19" ht="50" customHeight="1"/>
+    <row r="20" ht="100" customHeight="1">
       <c r="A20" s="81" t="inlineStr">
         <is>
           <t>Objetivo del documento</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="228" customHeight="1">
+    <row r="21" ht="300" customHeight="1">
       <c r="A21" s="86" t="inlineStr">
         <is>
           <t>Presentar de forma atómica, funcional y verificable el cálculo del caudal de aire, potencia del ventilador axial, área de impulsión del ventilador (sin ductos) y área/dimensiones de las rejillas de exfiltración para modelado CFD, con sustentación normativa.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="38" customHeight="1"/>
-    <row r="23" ht="38" customHeight="1"/>
-    <row r="24" ht="38" customHeight="1"/>
-    <row r="25" ht="76" customHeight="1">
+    <row r="22" ht="50" customHeight="1"/>
+    <row r="23" ht="50" customHeight="1"/>
+    <row r="24" ht="50" customHeight="1"/>
+    <row r="25" ht="100" customHeight="1">
       <c r="A25" s="81" t="inlineStr">
         <is>
           <t>2. PARÁMETROS DE ENTRADA</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="38" customHeight="1"/>
-    <row r="27" ht="76" customHeight="1">
+    <row r="26" ht="50" customHeight="1"/>
+    <row r="27" ht="100" customHeight="1">
       <c r="A27" s="82" t="inlineStr">
         <is>
           <t>Parámetro</t>
@@ -4402,7 +4402,7 @@
       <c r="N27" s="82" t="n"/>
       <c r="O27" s="82" t="n"/>
     </row>
-    <row r="28" ht="114" customHeight="1">
+    <row r="28" ht="150" customHeight="1">
       <c r="A28" s="83" t="inlineStr">
         <is>
           <t>Volumen efectivo del laboratorio</t>
@@ -4437,7 +4437,7 @@
       <c r="N28" s="84" t="n"/>
       <c r="O28" s="84" t="n"/>
     </row>
-    <row r="29" ht="76" customHeight="1">
+    <row r="29" ht="100" customHeight="1">
       <c r="A29" s="83" t="inlineStr">
         <is>
           <t>Renovaciones de aire</t>
@@ -4472,7 +4472,7 @@
       <c r="N29" s="84" t="n"/>
       <c r="O29" s="84" t="n"/>
     </row>
-    <row r="30" ht="190" customHeight="1">
+    <row r="30" ht="250" customHeight="1">
       <c r="A30" s="83" t="inlineStr">
         <is>
           <t>Presión total estimada del ventilador</t>
@@ -4507,7 +4507,7 @@
       <c r="N30" s="84" t="n"/>
       <c r="O30" s="84" t="n"/>
     </row>
-    <row r="31" ht="152" customHeight="1">
+    <row r="31" ht="200" customHeight="1">
       <c r="A31" s="83" t="inlineStr">
         <is>
           <t>Eficiencia total del ventilador</t>
@@ -4542,7 +4542,7 @@
       <c r="N31" s="84" t="n"/>
       <c r="O31" s="84" t="n"/>
     </row>
-    <row r="32" ht="114" customHeight="1">
+    <row r="32" ht="150" customHeight="1">
       <c r="A32" s="83" t="inlineStr">
         <is>
           <t>Velocidad en boca del ventilador</t>
@@ -4577,7 +4577,7 @@
       <c r="N32" s="84" t="n"/>
       <c r="O32" s="84" t="n"/>
     </row>
-    <row r="33" ht="114" customHeight="1">
+    <row r="33" ht="150" customHeight="1">
       <c r="A33" s="83" t="inlineStr">
         <is>
           <t>Velocidad de exfiltración en rejillas</t>
@@ -4612,7 +4612,7 @@
       <c r="N33" s="84" t="n"/>
       <c r="O33" s="84" t="n"/>
     </row>
-    <row r="34" ht="76" customHeight="1">
+    <row r="34" ht="100" customHeight="1">
       <c r="A34" s="83" t="inlineStr">
         <is>
           <t>Número de rejillas de salida</t>
@@ -4647,7 +4647,7 @@
       <c r="N34" s="84" t="n"/>
       <c r="O34" s="84" t="n"/>
     </row>
-    <row r="35" ht="114" customHeight="1">
+    <row r="35" ht="150" customHeight="1">
       <c r="A35" s="83" t="inlineStr">
         <is>
           <t>Proporción ancho/alto rejilla</t>
@@ -4682,7 +4682,7 @@
       <c r="N35" s="84" t="n"/>
       <c r="O35" s="84" t="n"/>
     </row>
-    <row r="36" ht="190" customHeight="1">
+    <row r="36" ht="250" customHeight="1">
       <c r="A36" s="83" t="inlineStr">
         <is>
           <t>Densidad del aire</t>
@@ -4717,7 +4717,7 @@
       <c r="N36" s="84" t="n"/>
       <c r="O36" s="84" t="n"/>
     </row>
-    <row r="37" ht="152" customHeight="1">
+    <row r="37" ht="200" customHeight="1">
       <c r="A37" s="83" t="inlineStr">
         <is>
           <t>Coeficiente de descarga orificio</t>
@@ -4752,45 +4752,45 @@
       <c r="N37" s="84" t="n"/>
       <c r="O37" s="84" t="n"/>
     </row>
-    <row r="38" ht="38" customHeight="1"/>
-    <row r="39" ht="38" customHeight="1">
+    <row r="38" ht="50" customHeight="1"/>
+    <row r="39" ht="50" customHeight="1">
       <c r="A39" s="81" t="inlineStr">
         <is>
           <t>Notas:</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="228" customHeight="1">
+    <row r="40" ht="300" customHeight="1">
       <c r="A40" s="86" t="inlineStr">
         <is>
           <t>• Modifique los valores en amarillo; todos los cálculos se actualizan automáticamente.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="190" customHeight="1">
+    <row r="41" ht="250" customHeight="1">
       <c r="A41" s="86" t="inlineStr">
         <is>
           <t>• Las fórmulas están visibles en la barra de fórmulas de cada celda.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="152" customHeight="1">
+    <row r="42" ht="200" customHeight="1">
       <c r="A42" s="86" t="inlineStr">
         <is>
           <t>• Unidades: 1 m³/min = 35.3147 CFM; 1 kW = 1.341 HP.</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="38" customHeight="1"/>
-    <row r="44" ht="76" customHeight="1">
+    <row r="43" ht="50" customHeight="1"/>
+    <row r="44" ht="100" customHeight="1">
       <c r="A44" s="81" t="inlineStr">
         <is>
           <t>3. DESARROLLO DE CÁLCULOS</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="38" customHeight="1"/>
-    <row r="46" ht="76" customHeight="1">
+    <row r="45" ht="50" customHeight="1"/>
+    <row r="46" ht="100" customHeight="1">
       <c r="A46" s="82" t="inlineStr">
         <is>
           <t>Paso</t>
@@ -4831,7 +4831,7 @@
       </c>
       <c r="O46" s="82" t="n"/>
     </row>
-    <row r="47" ht="76" customHeight="1">
+    <row r="47" ht="100" customHeight="1">
       <c r="A47" s="85" t="inlineStr">
         <is>
           <t>1</t>
@@ -4870,7 +4870,7 @@
       </c>
       <c r="O47" s="84" t="n"/>
     </row>
-    <row r="48" ht="76" customHeight="1">
+    <row r="48" ht="100" customHeight="1">
       <c r="A48" s="85" t="inlineStr">
         <is>
           <t>2</t>
@@ -4909,7 +4909,7 @@
       </c>
       <c r="O48" s="84" t="n"/>
     </row>
-    <row r="49" ht="76" customHeight="1">
+    <row r="49" ht="100" customHeight="1">
       <c r="A49" s="85" t="inlineStr">
         <is>
           <t>3</t>
@@ -4948,7 +4948,7 @@
       </c>
       <c r="O49" s="84" t="n"/>
     </row>
-    <row r="50" ht="38" customHeight="1">
+    <row r="50" ht="50" customHeight="1">
       <c r="A50" s="85" t="inlineStr">
         <is>
           <t>4</t>
@@ -4987,7 +4987,7 @@
       </c>
       <c r="O50" s="84" t="n"/>
     </row>
-    <row r="51" ht="114" customHeight="1">
+    <row r="51" ht="150" customHeight="1">
       <c r="A51" s="85" t="inlineStr">
         <is>
           <t>5</t>
@@ -5026,7 +5026,7 @@
       </c>
       <c r="O51" s="84" t="n"/>
     </row>
-    <row r="52" ht="38" customHeight="1">
+    <row r="52" ht="50" customHeight="1">
       <c r="A52" s="85" t="inlineStr">
         <is>
           <t>6</t>
@@ -5065,7 +5065,7 @@
       </c>
       <c r="O52" s="84" t="n"/>
     </row>
-    <row r="53" ht="114" customHeight="1">
+    <row r="53" ht="150" customHeight="1">
       <c r="A53" s="85" t="inlineStr">
         <is>
           <t>7</t>
@@ -5104,7 +5104,7 @@
       </c>
       <c r="O53" s="84" t="n"/>
     </row>
-    <row r="54" ht="114" customHeight="1">
+    <row r="54" ht="150" customHeight="1">
       <c r="A54" s="85" t="inlineStr">
         <is>
           <t>8</t>
@@ -5143,7 +5143,7 @@
       </c>
       <c r="O54" s="84" t="n"/>
     </row>
-    <row r="55" ht="76" customHeight="1">
+    <row r="55" ht="100" customHeight="1">
       <c r="A55" s="85" t="inlineStr">
         <is>
           <t>9</t>
@@ -5182,7 +5182,7 @@
       </c>
       <c r="O55" s="84" t="n"/>
     </row>
-    <row r="56" ht="76" customHeight="1">
+    <row r="56" ht="100" customHeight="1">
       <c r="A56" s="85" t="inlineStr">
         <is>
           <t>10</t>
@@ -5221,7 +5221,7 @@
       </c>
       <c r="O56" s="84" t="n"/>
     </row>
-    <row r="57" ht="114" customHeight="1">
+    <row r="57" ht="150" customHeight="1">
       <c r="A57" s="85" t="inlineStr">
         <is>
           <t>11</t>
@@ -5260,7 +5260,7 @@
       </c>
       <c r="O57" s="84" t="n"/>
     </row>
-    <row r="58" ht="114" customHeight="1">
+    <row r="58" ht="150" customHeight="1">
       <c r="A58" s="85" t="inlineStr">
         <is>
           <t>12</t>
@@ -5299,7 +5299,7 @@
       </c>
       <c r="O58" s="84" t="n"/>
     </row>
-    <row r="59" ht="114" customHeight="1">
+    <row r="59" ht="150" customHeight="1">
       <c r="A59" s="85" t="inlineStr">
         <is>
           <t>13</t>
@@ -5338,7 +5338,7 @@
       </c>
       <c r="O59" s="84" t="n"/>
     </row>
-    <row r="60" ht="76" customHeight="1">
+    <row r="60" ht="100" customHeight="1">
       <c r="A60" s="85" t="inlineStr">
         <is>
           <t>14</t>
@@ -5377,7 +5377,7 @@
       </c>
       <c r="O60" s="84" t="n"/>
     </row>
-    <row r="61" ht="76" customHeight="1">
+    <row r="61" ht="100" customHeight="1">
       <c r="A61" s="85" t="inlineStr">
         <is>
           <t>15</t>
@@ -5416,7 +5416,7 @@
       </c>
       <c r="O61" s="84" t="n"/>
     </row>
-    <row r="62" ht="76" customHeight="1">
+    <row r="62" ht="100" customHeight="1">
       <c r="A62" s="85" t="inlineStr">
         <is>
           <t>16</t>
@@ -5455,7 +5455,7 @@
       </c>
       <c r="O62" s="84" t="n"/>
     </row>
-    <row r="63" ht="152" customHeight="1">
+    <row r="63" ht="200" customHeight="1">
       <c r="A63" s="85" t="inlineStr">
         <is>
           <t>17</t>
@@ -5494,16 +5494,16 @@
       </c>
       <c r="O63" s="84" t="n"/>
     </row>
-    <row r="64" ht="38" customHeight="1"/>
-    <row r="65" ht="114" customHeight="1">
+    <row r="64" ht="50" customHeight="1"/>
+    <row r="65" ht="150" customHeight="1">
       <c r="A65" s="81" t="inlineStr">
         <is>
           <t>4. RESUMEN DE RESULTADOS DE DISEÑO</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="38" customHeight="1"/>
-    <row r="67" ht="38" customHeight="1">
+    <row r="66" ht="50" customHeight="1"/>
+    <row r="67" ht="50" customHeight="1">
       <c r="A67" s="82" t="inlineStr">
         <is>
           <t>Parámetro</t>
@@ -5536,7 +5536,7 @@
       <c r="N67" s="82" t="n"/>
       <c r="O67" s="82" t="n"/>
     </row>
-    <row r="68" ht="114" customHeight="1">
+    <row r="68" ht="150" customHeight="1">
       <c r="A68" s="83" t="inlineStr">
         <is>
           <t>Caudal de diseño</t>
@@ -5568,7 +5568,7 @@
       <c r="N68" s="84" t="n"/>
       <c r="O68" s="84" t="n"/>
     </row>
-    <row r="69" ht="114" customHeight="1">
+    <row r="69" ht="150" customHeight="1">
       <c r="A69" s="83" t="inlineStr">
         <is>
           <t>Caudal de diseño</t>
@@ -5600,7 +5600,7 @@
       <c r="N69" s="84" t="n"/>
       <c r="O69" s="84" t="n"/>
     </row>
-    <row r="70" ht="114" customHeight="1">
+    <row r="70" ht="150" customHeight="1">
       <c r="A70" s="83" t="inlineStr">
         <is>
           <t>Caudal de diseño</t>
@@ -5632,7 +5632,7 @@
       <c r="N70" s="84" t="n"/>
       <c r="O70" s="84" t="n"/>
     </row>
-    <row r="71" ht="152" customHeight="1">
+    <row r="71" ht="200" customHeight="1">
       <c r="A71" s="83" t="inlineStr">
         <is>
           <t>Potencia teórica del ventilador</t>
@@ -5664,7 +5664,7 @@
       <c r="N71" s="84" t="n"/>
       <c r="O71" s="84" t="n"/>
     </row>
-    <row r="72" ht="114" customHeight="1">
+    <row r="72" ht="150" customHeight="1">
       <c r="A72" s="83" t="inlineStr">
         <is>
           <t>Potencia teórica del ventilador</t>
@@ -5696,7 +5696,7 @@
       <c r="N72" s="84" t="n"/>
       <c r="O72" s="84" t="n"/>
     </row>
-    <row r="73" ht="228" customHeight="1">
+    <row r="73" ht="300" customHeight="1">
       <c r="A73" s="83" t="inlineStr">
         <is>
           <t>Potencia instalada recomendada</t>
@@ -5728,7 +5728,7 @@
       <c r="N73" s="84" t="n"/>
       <c r="O73" s="84" t="n"/>
     </row>
-    <row r="74" ht="114" customHeight="1">
+    <row r="74" ht="150" customHeight="1">
       <c r="A74" s="83" t="inlineStr">
         <is>
           <t>Área de impulsión del ventilador</t>
@@ -5760,7 +5760,7 @@
       <c r="N74" s="84" t="n"/>
       <c r="O74" s="84" t="n"/>
     </row>
-    <row r="75" ht="114" customHeight="1">
+    <row r="75" ht="150" customHeight="1">
       <c r="A75" s="83" t="inlineStr">
         <is>
           <t>Diámetro equivalente del ventilador</t>
@@ -5792,7 +5792,7 @@
       <c r="N75" s="84" t="n"/>
       <c r="O75" s="84" t="n"/>
     </row>
-    <row r="76" ht="152" customHeight="1">
+    <row r="76" ht="200" customHeight="1">
       <c r="A76" s="83" t="inlineStr">
         <is>
           <t>Radio del ventilador (CFD)</t>
@@ -5824,7 +5824,7 @@
       <c r="N76" s="84" t="n"/>
       <c r="O76" s="84" t="n"/>
     </row>
-    <row r="77" ht="152" customHeight="1">
+    <row r="77" ht="200" customHeight="1">
       <c r="A77" s="83" t="inlineStr">
         <is>
           <t>Diámetro del impulsor seleccionado</t>
@@ -5849,13 +5849,13 @@
       <c r="L77" s="84" t="n"/>
       <c r="M77" s="83" t="inlineStr">
         <is>
-          <t>Ø560 mm — uniformidad con montaje típico de planta (REV2)</t>
+          <t>Ø560 mm — uniformidad con montaje típico de planta</t>
         </is>
       </c>
       <c r="N77" s="84" t="n"/>
       <c r="O77" s="84" t="n"/>
     </row>
-    <row r="78" ht="76" customHeight="1">
+    <row r="78" ht="100" customHeight="1">
       <c r="A78" s="83" t="inlineStr">
         <is>
           <t>Área de boca real (Ø560 mm)</t>
@@ -5887,7 +5887,7 @@
       <c r="N78" s="84" t="n"/>
       <c r="O78" s="84" t="n"/>
     </row>
-    <row r="79" ht="114" customHeight="1">
+    <row r="79" ht="150" customHeight="1">
       <c r="A79" s="83" t="inlineStr">
         <is>
           <t>Velocidad real en boca (Ø560 mm)</t>
@@ -5919,7 +5919,7 @@
       <c r="N79" s="84" t="n"/>
       <c r="O79" s="84" t="n"/>
     </row>
-    <row r="80" ht="76" customHeight="1">
+    <row r="80" ht="100" customHeight="1">
       <c r="A80" s="83" t="inlineStr">
         <is>
           <t>Velocidad de impulsión</t>
@@ -5951,7 +5951,7 @@
       <c r="N80" s="84" t="n"/>
       <c r="O80" s="84" t="n"/>
     </row>
-    <row r="81" ht="114" customHeight="1">
+    <row r="81" ht="150" customHeight="1">
       <c r="A81" s="83" t="inlineStr">
         <is>
           <t>Área neta total de rejillas de salida</t>
@@ -5983,7 +5983,7 @@
       <c r="N81" s="84" t="n"/>
       <c r="O81" s="84" t="n"/>
     </row>
-    <row r="82" ht="76" customHeight="1">
+    <row r="82" ht="100" customHeight="1">
       <c r="A82" s="83" t="inlineStr">
         <is>
           <t>Número de rejillas de salida</t>
@@ -6015,7 +6015,7 @@
       <c r="N82" s="84" t="n"/>
       <c r="O82" s="84" t="n"/>
     </row>
-    <row r="83" ht="114" customHeight="1">
+    <row r="83" ht="150" customHeight="1">
       <c r="A83" s="83" t="inlineStr">
         <is>
           <t>Área neta por rejilla de salida</t>
@@ -6047,7 +6047,7 @@
       <c r="N83" s="84" t="n"/>
       <c r="O83" s="84" t="n"/>
     </row>
-    <row r="84" ht="76" customHeight="1">
+    <row r="84" ht="100" customHeight="1">
       <c r="A84" s="83" t="inlineStr">
         <is>
           <t>Altura de rejilla de salida</t>
@@ -6079,7 +6079,7 @@
       <c r="N84" s="84" t="n"/>
       <c r="O84" s="84" t="n"/>
     </row>
-    <row r="85" ht="76" customHeight="1">
+    <row r="85" ht="100" customHeight="1">
       <c r="A85" s="83" t="inlineStr">
         <is>
           <t>Ancho de rejilla de salida</t>
@@ -6111,7 +6111,7 @@
       <c r="N85" s="84" t="n"/>
       <c r="O85" s="84" t="n"/>
     </row>
-    <row r="86" ht="114" customHeight="1">
+    <row r="86" ht="150" customHeight="1">
       <c r="A86" s="83" t="inlineStr">
         <is>
           <t>Velocidad de exfiltración</t>
@@ -6143,7 +6143,7 @@
       <c r="N86" s="84" t="n"/>
       <c r="O86" s="84" t="n"/>
     </row>
-    <row r="87" ht="114" customHeight="1">
+    <row r="87" ht="150" customHeight="1">
       <c r="A87" s="83" t="inlineStr">
         <is>
           <t>Pérdida de presión en rejillas</t>
@@ -6175,16 +6175,16 @@
       <c r="N87" s="84" t="n"/>
       <c r="O87" s="84" t="n"/>
     </row>
-    <row r="88" ht="38" customHeight="1"/>
-    <row r="89" ht="152" customHeight="1">
+    <row r="88" ht="50" customHeight="1"/>
+    <row r="89" ht="200" customHeight="1">
       <c r="A89" s="81" t="inlineStr">
         <is>
           <t>5. SUSTENTACIÓN NORMATIVA — 12 RENOVACIONES/HORA</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="38" customHeight="1"/>
-    <row r="91" ht="76" customHeight="1">
+    <row r="90" ht="50" customHeight="1"/>
+    <row r="91" ht="100" customHeight="1">
       <c r="A91" s="82" t="inlineStr">
         <is>
           <t>Norma / Guía</t>
@@ -6217,7 +6217,7 @@
       <c r="N91" s="82" t="n"/>
       <c r="O91" s="82" t="n"/>
     </row>
-    <row r="92" ht="152" customHeight="1">
+    <row r="92" ht="200" customHeight="1">
       <c r="A92" s="83" t="inlineStr">
         <is>
           <t>ASHRAE 170 — Ventilation of Health Care Facilities</t>
@@ -6250,7 +6250,7 @@
       <c r="N92" s="84" t="n"/>
       <c r="O92" s="84" t="n"/>
     </row>
-    <row r="93" ht="152" customHeight="1">
+    <row r="93" ht="200" customHeight="1">
       <c r="A93" s="83" t="inlineStr">
         <is>
           <t>ASHRAE 62.1 — Ventilation for Acceptable IAQ</t>
@@ -6283,7 +6283,7 @@
       <c r="N93" s="84" t="n"/>
       <c r="O93" s="84" t="n"/>
     </row>
-    <row r="94" ht="114" customHeight="1">
+    <row r="94" ht="150" customHeight="1">
       <c r="A94" s="83" t="inlineStr">
         <is>
           <t>OSHA 29 CFR 1910.1450 — Laboratory Standard</t>
@@ -6316,7 +6316,7 @@
       <c r="N94" s="84" t="n"/>
       <c r="O94" s="84" t="n"/>
     </row>
-    <row r="95" ht="114" customHeight="1">
+    <row r="95" ht="150" customHeight="1">
       <c r="A95" s="83" t="inlineStr">
         <is>
           <t>NFPA 99 — Health Care Facilities Code</t>
@@ -6349,7 +6349,7 @@
       <c r="N95" s="84" t="n"/>
       <c r="O95" s="84" t="n"/>
     </row>
-    <row r="96" ht="114" customHeight="1">
+    <row r="96" ht="150" customHeight="1">
       <c r="A96" s="83" t="inlineStr">
         <is>
           <t>WHO — Laboratory Biosafety Manual (BSL-2)</t>
@@ -6382,7 +6382,7 @@
       <c r="N96" s="84" t="n"/>
       <c r="O96" s="84" t="n"/>
     </row>
-    <row r="97" ht="114" customHeight="1">
+    <row r="97" ht="150" customHeight="1">
       <c r="A97" s="83" t="inlineStr">
         <is>
           <t>WHO — Laboratory Biosafety Manual (BSL-3)</t>
@@ -6415,7 +6415,7 @@
       <c r="N97" s="84" t="n"/>
       <c r="O97" s="84" t="n"/>
     </row>
-    <row r="98" ht="152" customHeight="1">
+    <row r="98" ht="200" customHeight="1">
       <c r="A98" s="83" t="inlineStr">
         <is>
           <t>NIH — Design Requirements Manual</t>
@@ -6448,7 +6448,7 @@
       <c r="N98" s="84" t="n"/>
       <c r="O98" s="84" t="n"/>
     </row>
-    <row r="99" ht="114" customHeight="1">
+    <row r="99" ht="150" customHeight="1">
       <c r="A99" s="83" t="inlineStr">
         <is>
           <t>ASHRAE Handbook — Fundamentals</t>
@@ -6481,7 +6481,7 @@
       <c r="N99" s="84" t="n"/>
       <c r="O99" s="84" t="n"/>
     </row>
-    <row r="100" ht="152" customHeight="1">
+    <row r="100" ht="200" customHeight="1">
       <c r="A100" s="83" t="inlineStr">
         <is>
           <t>RETIE (Colombia)</t>
@@ -6514,7 +6514,7 @@
       <c r="N100" s="84" t="n"/>
       <c r="O100" s="84" t="n"/>
     </row>
-    <row r="101" ht="114" customHeight="1">
+    <row r="101" ht="150" customHeight="1">
       <c r="A101" s="83" t="inlineStr">
         <is>
           <t>NTC 2050 (Colombia)</t>
@@ -6547,7 +6547,7 @@
       <c r="N101" s="84" t="n"/>
       <c r="O101" s="84" t="n"/>
     </row>
-    <row r="102" ht="152" customHeight="1">
+    <row r="102" ht="200" customHeight="1">
       <c r="A102" s="83" t="inlineStr">
         <is>
           <t>Resolución 0312/2019 MinSalud (Colombia)</t>
@@ -6580,40 +6580,40 @@
       <c r="N102" s="84" t="n"/>
       <c r="O102" s="84" t="n"/>
     </row>
-    <row r="103" ht="38" customHeight="1"/>
-    <row r="104" ht="38" customHeight="1">
+    <row r="103" ht="50" customHeight="1"/>
+    <row r="104" ht="50" customHeight="1">
       <c r="A104" s="81" t="inlineStr">
         <is>
           <t>Conclusión</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="380" customHeight="1">
+    <row r="105" ht="500" customHeight="1">
       <c r="A105" s="86" t="inlineStr">
         <is>
           <t>La selección de 12 renovaciones de aire por hora está sustentada por las guías internacionales de bioseguridad (WHO BSL-2/BSL-3, NIH DRM) y los estándares de ventilación de ASHRAE para instalaciones de salud. El marco regulatorio local (RETIE, NTC 2050, Resolución 0312/2019) aplica a la infraestructura y seguridad eléctrica del equipo; no existe norma colombiana que fije un valor de ACH distinto para este caso.</t>
         </is>
       </c>
     </row>
-    <row r="106" ht="38" customHeight="1"/>
-    <row r="107" ht="38" customHeight="1"/>
-    <row r="108" ht="38" customHeight="1"/>
-    <row r="109" ht="152" customHeight="1">
+    <row r="106" ht="50" customHeight="1"/>
+    <row r="107" ht="50" customHeight="1"/>
+    <row r="108" ht="50" customHeight="1"/>
+    <row r="109" ht="200" customHeight="1">
       <c r="A109" s="81" t="inlineStr">
         <is>
           <t>6. ESCENARIOS DE FILTRACIÓN Y MOTOR RECOMENDADO</t>
         </is>
       </c>
     </row>
-    <row r="110" ht="608" customHeight="1">
+    <row r="110" ht="650" customHeight="1">
       <c r="A110" s="86" t="inlineStr">
         <is>
-          <t>ΔP_vent total = ΔP_filtro + ΔP_rejillas (11 Pa). Sin presurización (REV1: cambio de alcance del cliente). El caudal Q_s se toma del paso 4 de la sección 3 (celda J50). Sitio: Cajicá, Cundinamarca (2 558 msnm, ρ = 0.88 kg/m³).</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="38" customHeight="1"/>
-    <row r="112" ht="76" customHeight="1">
+          <t>ΔP_vent total = ΔP_filtro + ΔP_rejillas (11 Pa). Sin presurización. El caudal Q_s se toma del paso 4 de la sección 3 (celda J50). Sitio: Cajicá, Cundinamarca (2 558 msnm, ρ = 0.88 kg/m³).</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="50" customHeight="1"/>
+    <row r="112" ht="100" customHeight="1">
       <c r="A112" s="82" t="inlineStr">
         <is>
           <t>Escenario de filtración</t>
@@ -6654,7 +6654,7 @@
       </c>
       <c r="O112" s="82" t="n"/>
     </row>
-    <row r="113" ht="76" customHeight="1">
+    <row r="113" ht="100" customHeight="1">
       <c r="A113" s="83" t="inlineStr">
         <is>
           <t>MERV 13-14 limpio</t>
@@ -6689,7 +6689,7 @@
       </c>
       <c r="O113" s="94" t="n"/>
     </row>
-    <row r="114" ht="76" customHeight="1">
+    <row r="114" ht="100" customHeight="1">
       <c r="A114" s="83" t="inlineStr">
         <is>
           <t>MERV 13-14 cargado (diseño)</t>
@@ -6724,7 +6724,7 @@
       </c>
       <c r="O114" s="94" t="n"/>
     </row>
-    <row r="115" ht="152" customHeight="1">
+    <row r="115" ht="200" customHeight="1">
       <c r="A115" s="83" t="inlineStr">
         <is>
           <t>HEPA H13 limpio (referencia histórica — no aplica)</t>
@@ -6759,7 +6759,7 @@
       </c>
       <c r="O115" s="94" t="n"/>
     </row>
-    <row r="116" ht="152" customHeight="1">
+    <row r="116" ht="200" customHeight="1">
       <c r="A116" s="83" t="inlineStr">
         <is>
           <t>HEPA H13 cargado (referencia histórica — no aplica)</t>
@@ -6794,33 +6794,33 @@
       </c>
       <c r="O116" s="94" t="n"/>
     </row>
-    <row r="117" ht="38" customHeight="1"/>
-    <row r="118" ht="38" customHeight="1">
+    <row r="117" ht="50" customHeight="1"/>
+    <row r="118" ht="50" customHeight="1">
       <c r="A118" s="81" t="inlineStr">
         <is>
           <t>Nota:</t>
         </is>
       </c>
     </row>
-    <row r="119" ht="646" customHeight="1">
+    <row r="119" ht="850" customHeight="1">
       <c r="A119" s="86" t="inlineStr">
         <is>
-          <t>El motor provisional de 0.75 HP TEFC encapsulado anticorrosivo (en la corriente de aire, transmisión directa del ventilador mural Ø560 mm — uniformidad con el montaje típico de planta, REV2) corresponde al escenario MERV 13-14 cargado (punto de diseño), con margen de servicio 1.5 sobre la potencia teórica; la potencia definitiva se fija con la curva del ventilador axial seleccionado. Los escenarios HEPA son solo referencia histórica: el laboratorio de análisis industrial NO requiere HEPA. Para selección de ventilador en catálogo (ρ = 1.2 kg/m³), usar el punto equivalente 3 840 m³/h @ 225 Pa (diseño) o 95 Pa (limpio). La potencia se recalcula automáticamente si cambia el caudal en la sección 3. DESARROLLO DE CÁLCULOS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="120" ht="38" customHeight="1"/>
-    <row r="121" ht="38" customHeight="1"/>
-    <row r="122" ht="38" customHeight="1"/>
-    <row r="123" ht="152" customHeight="1">
+          <t>El motor provisional de 0.75 HP TEFC encapsulado anticorrosivo (en la corriente de aire, transmisión directa del ventilador mural Ø560 mm — uniformidad con el montaje típico de planta) corresponde al escenario MERV 13-14 cargado (punto de diseño), con margen de servicio 1.5 sobre la potencia teórica; la potencia definitiva se fija con la curva del ventilador axial seleccionado. Los escenarios HEPA son solo referencia histórica: el laboratorio de análisis industrial NO requiere HEPA. Para selección de ventilador en catálogo (ρ = 1.2 kg/m³), usar el punto equivalente 3 840 m³/h @ 225 Pa (diseño) o 95 Pa (limpio). La potencia se recalcula automáticamente si cambia el caudal en la sección 3. DESARROLLO DE CÁLCULOS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="50" customHeight="1"/>
+    <row r="121" ht="50" customHeight="1"/>
+    <row r="122" ht="50" customHeight="1"/>
+    <row r="123" ht="200" customHeight="1">
       <c r="A123" s="81" t="inlineStr">
         <is>
           <t>7. VISTA RÁPIDA — RESULTADOS (FÓRMULAS VIVAS)</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="38" customHeight="1"/>
-    <row r="125" ht="38" customHeight="1">
+    <row r="124" ht="50" customHeight="1"/>
+    <row r="125" ht="50" customHeight="1">
       <c r="A125" s="82" t="inlineStr">
         <is>
           <t>Parámetro</t>
@@ -6853,7 +6853,7 @@
       <c r="N125" s="82" t="n"/>
       <c r="O125" s="82" t="n"/>
     </row>
-    <row r="126" ht="114" customHeight="1">
+    <row r="126" ht="150" customHeight="1">
       <c r="A126" s="83" t="inlineStr">
         <is>
           <t>Caudal de diseño</t>
@@ -6885,7 +6885,7 @@
       <c r="N126" s="84" t="n"/>
       <c r="O126" s="84" t="n"/>
     </row>
-    <row r="127" ht="114" customHeight="1">
+    <row r="127" ht="150" customHeight="1">
       <c r="A127" s="83" t="inlineStr">
         <is>
           <t>Caudal de diseño</t>
@@ -6917,7 +6917,7 @@
       <c r="N127" s="84" t="n"/>
       <c r="O127" s="84" t="n"/>
     </row>
-    <row r="128" ht="114" customHeight="1">
+    <row r="128" ht="150" customHeight="1">
       <c r="A128" s="83" t="inlineStr">
         <is>
           <t>Caudal de diseño</t>
@@ -6949,7 +6949,7 @@
       <c r="N128" s="84" t="n"/>
       <c r="O128" s="84" t="n"/>
     </row>
-    <row r="129" ht="114" customHeight="1">
+    <row r="129" ht="150" customHeight="1">
       <c r="A129" s="83" t="inlineStr">
         <is>
           <t>Potencia teórica del ventilador</t>
@@ -6981,7 +6981,7 @@
       <c r="N129" s="84" t="n"/>
       <c r="O129" s="84" t="n"/>
     </row>
-    <row r="130" ht="114" customHeight="1">
+    <row r="130" ht="150" customHeight="1">
       <c r="A130" s="83" t="inlineStr">
         <is>
           <t>Potencia teórica del ventilador</t>
@@ -7013,7 +7013,7 @@
       <c r="N130" s="84" t="n"/>
       <c r="O130" s="84" t="n"/>
     </row>
-    <row r="131" ht="114" customHeight="1">
+    <row r="131" ht="150" customHeight="1">
       <c r="A131" s="83" t="inlineStr">
         <is>
           <t>Potencia instalada recomendada</t>
@@ -7045,7 +7045,7 @@
       <c r="N131" s="84" t="n"/>
       <c r="O131" s="84" t="n"/>
     </row>
-    <row r="132" ht="114" customHeight="1">
+    <row r="132" ht="150" customHeight="1">
       <c r="A132" s="83" t="inlineStr">
         <is>
           <t>Área de impulsión del ventilador</t>
@@ -7077,7 +7077,7 @@
       <c r="N132" s="84" t="n"/>
       <c r="O132" s="84" t="n"/>
     </row>
-    <row r="133" ht="114" customHeight="1">
+    <row r="133" ht="150" customHeight="1">
       <c r="A133" s="83" t="inlineStr">
         <is>
           <t>Diámetro equivalente del ventilador</t>
@@ -7109,7 +7109,7 @@
       <c r="N133" s="84" t="n"/>
       <c r="O133" s="84" t="n"/>
     </row>
-    <row r="134" ht="152" customHeight="1">
+    <row r="134" ht="200" customHeight="1">
       <c r="A134" s="83" t="inlineStr">
         <is>
           <t>Radio del ventilador (CFD)</t>
@@ -7141,7 +7141,7 @@
       <c r="N134" s="84" t="n"/>
       <c r="O134" s="84" t="n"/>
     </row>
-    <row r="135" ht="152" customHeight="1">
+    <row r="135" ht="200" customHeight="1">
       <c r="A135" s="83" t="inlineStr">
         <is>
           <t>Diámetro del impulsor seleccionado</t>
@@ -7166,13 +7166,13 @@
       <c r="L135" s="84" t="n"/>
       <c r="M135" s="83" t="inlineStr">
         <is>
-          <t>Ø560 mm — uniformidad con montaje típico de planta (REV2)</t>
+          <t>Ø560 mm — uniformidad con montaje típico de planta</t>
         </is>
       </c>
       <c r="N135" s="84" t="n"/>
       <c r="O135" s="84" t="n"/>
     </row>
-    <row r="136" ht="76" customHeight="1">
+    <row r="136" ht="100" customHeight="1">
       <c r="A136" s="83" t="inlineStr">
         <is>
           <t>Área de boca real (Ø560 mm)</t>
@@ -7204,7 +7204,7 @@
       <c r="N136" s="84" t="n"/>
       <c r="O136" s="84" t="n"/>
     </row>
-    <row r="137" ht="114" customHeight="1">
+    <row r="137" ht="150" customHeight="1">
       <c r="A137" s="83" t="inlineStr">
         <is>
           <t>Velocidad real en boca (Ø560 mm)</t>
@@ -7236,7 +7236,7 @@
       <c r="N137" s="84" t="n"/>
       <c r="O137" s="84" t="n"/>
     </row>
-    <row r="138" ht="76" customHeight="1">
+    <row r="138" ht="100" customHeight="1">
       <c r="A138" s="83" t="inlineStr">
         <is>
           <t>Velocidad de impulsión</t>
@@ -7268,7 +7268,7 @@
       <c r="N138" s="84" t="n"/>
       <c r="O138" s="84" t="n"/>
     </row>
-    <row r="139" ht="114" customHeight="1">
+    <row r="139" ht="150" customHeight="1">
       <c r="A139" s="83" t="inlineStr">
         <is>
           <t>Área neta total de rejillas de salida</t>
@@ -7300,7 +7300,7 @@
       <c r="N139" s="84" t="n"/>
       <c r="O139" s="84" t="n"/>
     </row>
-    <row r="140" ht="76" customHeight="1">
+    <row r="140" ht="100" customHeight="1">
       <c r="A140" s="83" t="inlineStr">
         <is>
           <t>Número de rejillas de salida</t>
@@ -7332,7 +7332,7 @@
       <c r="N140" s="84" t="n"/>
       <c r="O140" s="84" t="n"/>
     </row>
-    <row r="141" ht="114" customHeight="1">
+    <row r="141" ht="150" customHeight="1">
       <c r="A141" s="83" t="inlineStr">
         <is>
           <t>Área neta por rejilla de salida</t>
@@ -7364,7 +7364,7 @@
       <c r="N141" s="84" t="n"/>
       <c r="O141" s="84" t="n"/>
     </row>
-    <row r="142" ht="76" customHeight="1">
+    <row r="142" ht="100" customHeight="1">
       <c r="A142" s="83" t="inlineStr">
         <is>
           <t>Altura de rejilla de salida</t>
@@ -7396,7 +7396,7 @@
       <c r="N142" s="84" t="n"/>
       <c r="O142" s="84" t="n"/>
     </row>
-    <row r="143" ht="76" customHeight="1">
+    <row r="143" ht="100" customHeight="1">
       <c r="A143" s="83" t="inlineStr">
         <is>
           <t>Ancho de rejilla de salida</t>
@@ -7428,7 +7428,7 @@
       <c r="N143" s="84" t="n"/>
       <c r="O143" s="84" t="n"/>
     </row>
-    <row r="144" ht="76" customHeight="1">
+    <row r="144" ht="100" customHeight="1">
       <c r="A144" s="83" t="inlineStr">
         <is>
           <t>Velocidad de exfiltración</t>
@@ -7460,7 +7460,7 @@
       <c r="N144" s="84" t="n"/>
       <c r="O144" s="84" t="n"/>
     </row>
-    <row r="145" ht="114" customHeight="1">
+    <row r="145" ht="150" customHeight="1">
       <c r="A145" s="83" t="inlineStr">
         <is>
           <t>Pérdida de presión en rejillas</t>
@@ -7492,23 +7492,23 @@
       <c r="N145" s="84" t="n"/>
       <c r="O145" s="84" t="n"/>
     </row>
-    <row r="146" ht="38" customHeight="1"/>
-    <row r="147" ht="38" customHeight="1">
+    <row r="146" ht="50" customHeight="1"/>
+    <row r="147" ht="50" customHeight="1">
       <c r="A147" s="81" t="inlineStr">
         <is>
           <t>Nota:</t>
         </is>
       </c>
     </row>
-    <row r="148" ht="228" customHeight="1">
+    <row r="148" ht="300" customHeight="1">
       <c r="A148" s="86" t="inlineStr">
         <is>
           <t>Sección con fórmulas vivas que referencian las secciones 3. DESARROLLO DE CÁLCULOS y 2. PARÁMETROS DE ENTRADA de esta misma hoja. Si modifica las entradas, esta vista y la sección 4. RESULTADOS se actualizan automáticamente.</t>
         </is>
       </c>
     </row>
-    <row r="149" ht="38" customHeight="1"/>
-    <row r="150" ht="38" customHeight="1"/>
+    <row r="149" ht="50" customHeight="1"/>
+    <row r="150" ht="50" customHeight="1"/>
   </sheetData>
   <mergeCells count="469">
     <mergeCell ref="A25:O25"/>

</xml_diff>